<commit_message>
vault backup: 2026-06-11 10:38:12
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -510,7 +510,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -544,12 +544,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -913,7 +907,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -937,16 +931,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -955,85 +949,85 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1077,7 +1071,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
vault backup: 2026-06-11 10:45:45
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15020"/>
+    <workbookView windowHeight="15020" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -3846,6 +3846,8 @@
     <col min="8" max="8" width="15.1538461538462" customWidth="1"/>
     <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
+    <col min="13" max="13" width="22.4615384615385" customWidth="1"/>
+    <col min="17" max="17" width="18.6923076923077" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">

</xml_diff>

<commit_message>
vault backup: 2026-06-11 11:09:06
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15020" activeTab="2"/>
+    <workbookView windowHeight="15020" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="106">
   <si>
     <t>招标方式</t>
   </si>
@@ -175,6 +175,9 @@
     <t>联系电话</t>
   </si>
   <si>
+    <t>询比采购（公开）</t>
+  </si>
+  <si>
     <t>标段/包件名称</t>
   </si>
   <si>
@@ -292,7 +295,7 @@
     <t>默认选择不允许</t>
   </si>
   <si>
-    <t>工期(天)/服务期（天）/</t>
+    <t>工期(天)/服务期（天）/交货期（天）</t>
   </si>
   <si>
     <t>是否两阶段项目</t>
@@ -301,7 +304,7 @@
     <t>默认选择否</t>
   </si>
   <si>
-    <t>工期说明/服务期说明</t>
+    <t>工期说明/服务期说明/交货期说明</t>
   </si>
   <si>
     <t>招标/采购范围</t>
@@ -3846,7 +3849,9 @@
     <col min="8" max="8" width="15.1538461538462" customWidth="1"/>
     <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
+    <col min="11" max="12" width="20" customWidth="1"/>
     <col min="13" max="13" width="22.4615384615385" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
     <col min="17" max="17" width="18.6923076923077" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3880,16 +3885,16 @@
         <v>2</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="O1" s="8" t="s">
         <v>4</v>
@@ -4010,10 +4015,10 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
@@ -4078,10 +4083,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
@@ -4146,10 +4151,10 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
@@ -4214,10 +4219,10 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -4276,7 +4281,7 @@
         <v>1</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Z6" s="7">
         <v>1</v>
@@ -4284,10 +4289,10 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
@@ -4352,10 +4357,10 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="2">
         <v>1</v>
@@ -4404,7 +4409,7 @@
         <v>1</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="V8" s="9">
         <v>1</v>
@@ -4422,10 +4427,10 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>20</v>
@@ -4454,7 +4459,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N9" s="7">
         <v>1</v>
@@ -4466,7 +4471,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="R9" s="8">
         <v>1</v>
@@ -4478,7 +4483,7 @@
         <v>1</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
@@ -4496,10 +4501,10 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>20</v>
@@ -4528,7 +4533,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N10" s="7">
         <v>1</v>
@@ -4540,31 +4545,31 @@
         <v>1</v>
       </c>
       <c r="Q10" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="R10" s="8">
+        <v>1</v>
+      </c>
+      <c r="S10" s="9">
+        <v>1</v>
+      </c>
+      <c r="T10" s="9">
+        <v>1</v>
+      </c>
+      <c r="U10" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="V10" s="9">
+        <v>0</v>
+      </c>
+      <c r="W10" s="7">
+        <v>1</v>
+      </c>
+      <c r="X10" s="7">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="R10" s="8">
-        <v>1</v>
-      </c>
-      <c r="S10" s="9">
-        <v>1</v>
-      </c>
-      <c r="T10" s="9">
-        <v>1</v>
-      </c>
-      <c r="U10" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="V10" s="9">
-        <v>0</v>
-      </c>
-      <c r="W10" s="7">
-        <v>1</v>
-      </c>
-      <c r="X10" s="7">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="7" t="s">
-        <v>62</v>
       </c>
       <c r="Z10" s="7">
         <v>0</v>
@@ -4572,10 +4577,10 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>20</v>
@@ -4604,7 +4609,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N11" s="7">
         <v>0</v>
@@ -4616,7 +4621,7 @@
         <v>1</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="R11" s="8">
         <v>0</v>
@@ -4644,10 +4649,10 @@
     </row>
     <row r="12" spans="1:26">
       <c r="A12" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>20</v>
@@ -4706,7 +4711,7 @@
         <v>1</v>
       </c>
       <c r="Y12" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Z12" s="7">
         <v>1</v>
@@ -4714,10 +4719,10 @@
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>20</v>
@@ -4776,7 +4781,7 @@
         <v>1</v>
       </c>
       <c r="Y13" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Z13" s="7">
         <v>0</v>
@@ -4784,10 +4789,10 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>20</v>
@@ -4816,7 +4821,7 @@
         <v>1</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N14" s="7">
         <v>0</v>
@@ -4828,7 +4833,7 @@
         <v>1</v>
       </c>
       <c r="Q14" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R14" s="8">
         <v>0</v>
@@ -4850,7 +4855,7 @@
         <v>1</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Z14" s="7">
         <v>1</v>
@@ -4858,10 +4863,10 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -4926,10 +4931,10 @@
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -4994,10 +4999,10 @@
     </row>
     <row r="17" spans="1:26">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C17" s="2">
         <v>1</v>
@@ -5026,7 +5031,7 @@
         <v>1</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N17" s="7">
         <v>1</v>
@@ -5064,10 +5069,10 @@
     </row>
     <row r="18" spans="1:26">
       <c r="A18" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -5132,10 +5137,10 @@
     </row>
     <row r="19" spans="1:26">
       <c r="A19" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>20</v>
@@ -5200,10 +5205,10 @@
     </row>
     <row r="20" spans="1:26">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>20</v>
@@ -5268,10 +5273,10 @@
     </row>
     <row r="21" ht="17" spans="1:26">
       <c r="A21" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>20</v>
@@ -5336,10 +5341,10 @@
     </row>
     <row r="22" spans="1:26">
       <c r="A22" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>20</v>
@@ -5404,10 +5409,10 @@
     </row>
     <row r="23" spans="1:26">
       <c r="A23" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>20</v>
@@ -5472,10 +5477,10 @@
     </row>
     <row r="24" spans="1:26">
       <c r="A24" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>20</v>
@@ -5540,10 +5545,10 @@
     </row>
     <row r="25" spans="1:26">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -5552,7 +5557,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F25" s="4">
         <v>1</v>
@@ -5610,10 +5615,10 @@
     </row>
     <row r="26" spans="1:26">
       <c r="A26" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>
@@ -5678,10 +5683,10 @@
     </row>
     <row r="27" spans="1:26">
       <c r="A27" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C27" s="2">
         <v>0</v>
@@ -5690,7 +5695,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F27" s="4">
         <v>1</v>
@@ -5748,10 +5753,10 @@
     </row>
     <row r="28" spans="1:26">
       <c r="A28" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" s="2">
         <v>1</v>
@@ -5816,10 +5821,10 @@
     </row>
     <row r="29" spans="1:26">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C29" s="2">
         <v>1</v>
@@ -5884,7 +5889,7 @@
     </row>
     <row r="30" spans="1:26">
       <c r="A30" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>36</v>
@@ -5950,10 +5955,10 @@
     </row>
     <row r="31" spans="1:26">
       <c r="A31" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C31" s="2">
         <v>1</v>
@@ -6018,10 +6023,10 @@
     </row>
     <row r="32" spans="1:26">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C32" s="2">
         <v>1</v>
@@ -6086,10 +6091,10 @@
     </row>
     <row r="33" spans="1:26">
       <c r="A33" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C33" s="2">
         <v>1</v>
@@ -6154,10 +6159,10 @@
     </row>
     <row r="34" spans="1:26">
       <c r="A34" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C34" s="2">
         <v>0</v>
@@ -6222,13 +6227,13 @@
     </row>
     <row r="35" spans="1:26">
       <c r="A35" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D35" s="3">
         <v>1</v>
@@ -6238,7 +6243,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H35" s="5">
         <v>1</v>
@@ -6290,10 +6295,10 @@
     </row>
     <row r="36" ht="34" spans="1:26">
       <c r="A36" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C36" s="2">
         <v>1</v>
@@ -6528,10 +6533,10 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>20</v>
@@ -6574,7 +6579,7 @@
         <v>1</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V3" s="9">
         <v>0</v>
@@ -6592,10 +6597,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -6654,10 +6659,10 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>20</v>
@@ -6716,10 +6721,10 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -6778,7 +6783,7 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
vault backup: 2026-06-11 11:10:56
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="107">
   <si>
     <t>招标方式</t>
   </si>
@@ -200,6 +200,9 @@
   </si>
   <si>
     <t>评审办法</t>
+  </si>
+  <si>
+    <t>默认填充经评审的最低投标价法</t>
   </si>
   <si>
     <t>经评审的最低投标价法</t>
@@ -3850,7 +3853,7 @@
     <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
     <col min="11" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="22.4615384615385" customWidth="1"/>
+    <col min="13" max="13" width="34.5384615384615" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
     <col min="17" max="17" width="18.6923076923077" customWidth="1"/>
   </cols>
@@ -4386,9 +4389,11 @@
         <v>1</v>
       </c>
       <c r="L8" s="7">
-        <v>0</v>
-      </c>
-      <c r="M8" s="7"/>
+        <v>1</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>57</v>
+      </c>
       <c r="N8" s="7">
         <v>1</v>
       </c>
@@ -4409,7 +4414,7 @@
         <v>1</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V8" s="9">
         <v>1</v>
@@ -4430,7 +4435,7 @@
         <v>49</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>20</v>
@@ -4459,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="N9" s="7">
         <v>1</v>
@@ -4471,7 +4476,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="R9" s="8">
         <v>1</v>
@@ -4483,7 +4488,7 @@
         <v>1</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="V9" s="9">
         <v>1</v>
@@ -4504,7 +4509,7 @@
         <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>20</v>
@@ -4533,7 +4538,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N10" s="7">
         <v>1</v>
@@ -4545,31 +4550,31 @@
         <v>1</v>
       </c>
       <c r="Q10" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="R10" s="8">
+        <v>1</v>
+      </c>
+      <c r="S10" s="9">
+        <v>1</v>
+      </c>
+      <c r="T10" s="9">
+        <v>1</v>
+      </c>
+      <c r="U10" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="V10" s="9">
+        <v>0</v>
+      </c>
+      <c r="W10" s="7">
+        <v>1</v>
+      </c>
+      <c r="X10" s="7">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="7" t="s">
         <v>64</v>
-      </c>
-      <c r="R10" s="8">
-        <v>1</v>
-      </c>
-      <c r="S10" s="9">
-        <v>1</v>
-      </c>
-      <c r="T10" s="9">
-        <v>1</v>
-      </c>
-      <c r="U10" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="V10" s="9">
-        <v>0</v>
-      </c>
-      <c r="W10" s="7">
-        <v>1</v>
-      </c>
-      <c r="X10" s="7">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="7" t="s">
-        <v>63</v>
       </c>
       <c r="Z10" s="7">
         <v>0</v>
@@ -4580,7 +4585,7 @@
         <v>49</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>20</v>
@@ -4609,7 +4614,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N11" s="7">
         <v>0</v>
@@ -4621,7 +4626,7 @@
         <v>1</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R11" s="8">
         <v>0</v>
@@ -4652,7 +4657,7 @@
         <v>49</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>20</v>
@@ -4711,7 +4716,7 @@
         <v>1</v>
       </c>
       <c r="Y12" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Z12" s="7">
         <v>1</v>
@@ -4722,7 +4727,7 @@
         <v>49</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>20</v>
@@ -4781,7 +4786,7 @@
         <v>1</v>
       </c>
       <c r="Y13" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Z13" s="7">
         <v>0</v>
@@ -4792,7 +4797,7 @@
         <v>49</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>20</v>
@@ -4821,7 +4826,7 @@
         <v>1</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N14" s="7">
         <v>0</v>
@@ -4833,7 +4838,7 @@
         <v>1</v>
       </c>
       <c r="Q14" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R14" s="8">
         <v>0</v>
@@ -4855,7 +4860,7 @@
         <v>1</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Z14" s="7">
         <v>1</v>
@@ -4866,7 +4871,7 @@
         <v>49</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -4934,7 +4939,7 @@
         <v>49</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -5002,7 +5007,7 @@
         <v>49</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C17" s="2">
         <v>1</v>
@@ -5031,7 +5036,7 @@
         <v>1</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N17" s="7">
         <v>1</v>
@@ -5072,7 +5077,7 @@
         <v>49</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -5140,7 +5145,7 @@
         <v>49</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>20</v>
@@ -5208,7 +5213,7 @@
         <v>49</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>20</v>
@@ -5276,7 +5281,7 @@
         <v>49</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>20</v>
@@ -5344,7 +5349,7 @@
         <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>20</v>
@@ -5412,7 +5417,7 @@
         <v>49</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>20</v>
@@ -5480,7 +5485,7 @@
         <v>49</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>20</v>
@@ -5548,7 +5553,7 @@
         <v>49</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -5557,7 +5562,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F25" s="4">
         <v>1</v>
@@ -5618,7 +5623,7 @@
         <v>49</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>
@@ -5686,7 +5691,7 @@
         <v>49</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C27" s="2">
         <v>0</v>
@@ -5695,7 +5700,7 @@
         <v>1</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F27" s="4">
         <v>1</v>
@@ -5756,7 +5761,7 @@
         <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C28" s="2">
         <v>1</v>
@@ -5824,7 +5829,7 @@
         <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C29" s="2">
         <v>1</v>
@@ -5958,7 +5963,7 @@
         <v>49</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C31" s="2">
         <v>1</v>
@@ -6026,7 +6031,7 @@
         <v>49</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C32" s="2">
         <v>1</v>
@@ -6094,7 +6099,7 @@
         <v>49</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C33" s="2">
         <v>1</v>
@@ -6162,7 +6167,7 @@
         <v>49</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C34" s="2">
         <v>0</v>
@@ -6230,10 +6235,10 @@
         <v>49</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D35" s="3">
         <v>1</v>
@@ -6243,7 +6248,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H35" s="5">
         <v>1</v>
@@ -6298,7 +6303,7 @@
         <v>49</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C36" s="2">
         <v>1</v>
@@ -6533,10 +6538,10 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>20</v>
@@ -6579,7 +6584,7 @@
         <v>1</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="V3" s="9">
         <v>0</v>
@@ -6597,10 +6602,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -6659,10 +6664,10 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>20</v>
@@ -6721,10 +6726,10 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -6783,7 +6788,7 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
vault backup: 2026-06-11 11:12:10
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15020" activeTab="1"/>
+    <workbookView windowHeight="15020" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="108">
   <si>
     <t>招标方式</t>
   </si>
@@ -333,6 +333,9 @@
   <si>
     <t xml:space="preserve">供应商其他要求
 </t>
+  </si>
+  <si>
+    <t>询比采购（邀请）</t>
   </si>
   <si>
     <t>邀请供应商</t>
@@ -516,7 +519,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,6 +541,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -913,7 +922,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -937,16 +946,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -955,89 +964,89 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1066,6 +1075,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1610,22 +1631,22 @@
   <cols>
     <col min="1" max="1" width="16.3846153846154" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="22.4615384615385" style="11" customWidth="1"/>
-    <col min="4" max="5" width="15.1538461538462" style="11" customWidth="1"/>
-    <col min="6" max="6" width="12.7692307692308" style="11" customWidth="1"/>
-    <col min="7" max="7" width="22.4615384615385" style="12" customWidth="1"/>
-    <col min="8" max="9" width="15.1538461538462" style="12" customWidth="1"/>
-    <col min="10" max="10" width="10.3076923076923" style="12" customWidth="1"/>
-    <col min="11" max="11" width="10.3076923076923" style="11" customWidth="1"/>
-    <col min="12" max="12" width="15.1538461538462" style="11" customWidth="1"/>
-    <col min="13" max="13" width="22.4615384615385" style="11" customWidth="1"/>
-    <col min="14" max="14" width="12.7692307692308" style="11" customWidth="1"/>
-    <col min="15" max="16" width="15.1538461538462" style="11" customWidth="1"/>
-    <col min="17" max="17" width="18.6923076923077" style="11" customWidth="1"/>
-    <col min="18" max="18" width="12.7692307692308" style="11" customWidth="1"/>
-    <col min="19" max="20" width="15.1538461538462" style="11" customWidth="1"/>
-    <col min="21" max="21" width="24.8461538461538" style="11" customWidth="1"/>
-    <col min="22" max="22" width="12.7692307692308" style="11" customWidth="1"/>
+    <col min="3" max="3" width="22.4615384615385" style="15" customWidth="1"/>
+    <col min="4" max="5" width="15.1538461538462" style="15" customWidth="1"/>
+    <col min="6" max="6" width="12.7692307692308" style="15" customWidth="1"/>
+    <col min="7" max="7" width="22.4615384615385" style="16" customWidth="1"/>
+    <col min="8" max="9" width="15.1538461538462" style="16" customWidth="1"/>
+    <col min="10" max="10" width="10.3076923076923" style="16" customWidth="1"/>
+    <col min="11" max="11" width="10.3076923076923" style="15" customWidth="1"/>
+    <col min="12" max="12" width="15.1538461538462" style="15" customWidth="1"/>
+    <col min="13" max="13" width="22.4615384615385" style="15" customWidth="1"/>
+    <col min="14" max="14" width="12.7692307692308" style="15" customWidth="1"/>
+    <col min="15" max="16" width="15.1538461538462" style="15" customWidth="1"/>
+    <col min="17" max="17" width="18.6923076923077" style="15" customWidth="1"/>
+    <col min="18" max="18" width="12.7692307692308" style="15" customWidth="1"/>
+    <col min="19" max="20" width="15.1538461538462" style="15" customWidth="1"/>
+    <col min="21" max="21" width="24.8461538461538" style="15" customWidth="1"/>
+    <col min="22" max="22" width="12.7692307692308" style="15" customWidth="1"/>
     <col min="23" max="23" width="10.3076923076923" customWidth="1"/>
     <col min="24" max="24" width="15.1538461538462" customWidth="1"/>
     <col min="25" max="25" width="41.8461538461538" customWidth="1"/>
@@ -1673,28 +1694,28 @@
       <c r="N1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="10" t="s">
         <v>5</v>
       </c>
       <c r="W1" s="7" t="s">
@@ -1753,28 +1774,28 @@
       <c r="N2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="P2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="R2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="T2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="V2" s="9" t="s">
+      <c r="V2" s="10" t="s">
         <v>12</v>
       </c>
       <c r="W2" s="7" t="s">
@@ -1827,24 +1848,24 @@
       <c r="N3" s="7">
         <v>0</v>
       </c>
-      <c r="O3" s="8">
-        <v>1</v>
-      </c>
-      <c r="P3" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8">
-        <v>0</v>
-      </c>
-      <c r="S3" s="9">
-        <v>1</v>
-      </c>
-      <c r="T3" s="9">
-        <v>0</v>
-      </c>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9">
+      <c r="O3" s="9">
+        <v>1</v>
+      </c>
+      <c r="P3" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9">
+        <v>0</v>
+      </c>
+      <c r="S3" s="10">
+        <v>1</v>
+      </c>
+      <c r="T3" s="10">
+        <v>0</v>
+      </c>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10">
         <v>0</v>
       </c>
       <c r="W3" s="7">
@@ -1895,24 +1916,24 @@
       <c r="N4" s="7">
         <v>0</v>
       </c>
-      <c r="O4" s="8">
-        <v>0</v>
-      </c>
-      <c r="P4" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8">
-        <v>0</v>
-      </c>
-      <c r="S4" s="9">
-        <v>0</v>
-      </c>
-      <c r="T4" s="9">
-        <v>1</v>
-      </c>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9">
+      <c r="O4" s="9">
+        <v>0</v>
+      </c>
+      <c r="P4" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9">
+        <v>0</v>
+      </c>
+      <c r="S4" s="10">
+        <v>0</v>
+      </c>
+      <c r="T4" s="10">
+        <v>1</v>
+      </c>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10">
         <v>0</v>
       </c>
       <c r="W4" s="7">
@@ -1963,24 +1984,24 @@
       <c r="N5" s="7">
         <v>0</v>
       </c>
-      <c r="O5" s="8">
-        <v>0</v>
-      </c>
-      <c r="P5" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8">
-        <v>0</v>
-      </c>
-      <c r="S5" s="9">
-        <v>0</v>
-      </c>
-      <c r="T5" s="9">
-        <v>1</v>
-      </c>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9">
+      <c r="O5" s="9">
+        <v>0</v>
+      </c>
+      <c r="P5" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9">
+        <v>0</v>
+      </c>
+      <c r="S5" s="10">
+        <v>0</v>
+      </c>
+      <c r="T5" s="10">
+        <v>1</v>
+      </c>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10">
         <v>0</v>
       </c>
       <c r="W5" s="7">
@@ -2031,24 +2052,24 @@
       <c r="N6" s="7">
         <v>1</v>
       </c>
-      <c r="O6" s="8">
-        <v>1</v>
-      </c>
-      <c r="P6" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8">
-        <v>1</v>
-      </c>
-      <c r="S6" s="9">
-        <v>1</v>
-      </c>
-      <c r="T6" s="9">
-        <v>1</v>
-      </c>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9">
+      <c r="O6" s="9">
+        <v>1</v>
+      </c>
+      <c r="P6" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9">
+        <v>1</v>
+      </c>
+      <c r="S6" s="10">
+        <v>1</v>
+      </c>
+      <c r="T6" s="10">
+        <v>1</v>
+      </c>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10">
         <v>1</v>
       </c>
       <c r="W6" s="7">
@@ -2099,24 +2120,24 @@
       <c r="N7" s="7">
         <v>0</v>
       </c>
-      <c r="O7" s="8">
-        <v>0</v>
-      </c>
-      <c r="P7" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8">
-        <v>0</v>
-      </c>
-      <c r="S7" s="9">
-        <v>0</v>
-      </c>
-      <c r="T7" s="9">
-        <v>1</v>
-      </c>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9">
+      <c r="O7" s="9">
+        <v>0</v>
+      </c>
+      <c r="P7" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9">
+        <v>0</v>
+      </c>
+      <c r="S7" s="10">
+        <v>0</v>
+      </c>
+      <c r="T7" s="10">
+        <v>1</v>
+      </c>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10">
         <v>0</v>
       </c>
       <c r="W7" s="7">
@@ -2167,24 +2188,24 @@
       <c r="N8" s="7">
         <v>1</v>
       </c>
-      <c r="O8" s="8">
-        <v>0</v>
-      </c>
-      <c r="P8" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8">
-        <v>1</v>
-      </c>
-      <c r="S8" s="9">
-        <v>0</v>
-      </c>
-      <c r="T8" s="9">
-        <v>1</v>
-      </c>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9">
+      <c r="O8" s="9">
+        <v>0</v>
+      </c>
+      <c r="P8" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9">
+        <v>1</v>
+      </c>
+      <c r="S8" s="10">
+        <v>0</v>
+      </c>
+      <c r="T8" s="10">
+        <v>1</v>
+      </c>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10">
         <v>1</v>
       </c>
       <c r="W8" s="7" t="s">
@@ -2235,24 +2256,24 @@
       <c r="N9" s="7">
         <v>1</v>
       </c>
-      <c r="O9" s="8">
-        <v>0</v>
-      </c>
-      <c r="P9" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="8">
-        <v>1</v>
-      </c>
-      <c r="S9" s="9">
-        <v>0</v>
-      </c>
-      <c r="T9" s="9">
-        <v>1</v>
-      </c>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9">
+      <c r="O9" s="9">
+        <v>0</v>
+      </c>
+      <c r="P9" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9">
+        <v>1</v>
+      </c>
+      <c r="S9" s="10">
+        <v>0</v>
+      </c>
+      <c r="T9" s="10">
+        <v>1</v>
+      </c>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10">
         <v>1</v>
       </c>
       <c r="W9" s="7" t="s">
@@ -2303,24 +2324,24 @@
       <c r="N10" s="7">
         <v>0</v>
       </c>
-      <c r="O10" s="8">
-        <v>0</v>
-      </c>
-      <c r="P10" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8">
-        <v>0</v>
-      </c>
-      <c r="S10" s="9">
-        <v>0</v>
-      </c>
-      <c r="T10" s="9">
-        <v>1</v>
-      </c>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9">
+      <c r="O10" s="9">
+        <v>0</v>
+      </c>
+      <c r="P10" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9">
+        <v>0</v>
+      </c>
+      <c r="S10" s="10">
+        <v>0</v>
+      </c>
+      <c r="T10" s="10">
+        <v>1</v>
+      </c>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10">
         <v>0</v>
       </c>
       <c r="W10" s="7">
@@ -2371,24 +2392,24 @@
       <c r="N11" s="7">
         <v>1</v>
       </c>
-      <c r="O11" s="8">
-        <v>0</v>
-      </c>
-      <c r="P11" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="8">
-        <v>1</v>
-      </c>
-      <c r="S11" s="9">
-        <v>0</v>
-      </c>
-      <c r="T11" s="9">
-        <v>1</v>
-      </c>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9">
+      <c r="O11" s="9">
+        <v>0</v>
+      </c>
+      <c r="P11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9">
+        <v>1</v>
+      </c>
+      <c r="S11" s="10">
+        <v>0</v>
+      </c>
+      <c r="T11" s="10">
+        <v>1</v>
+      </c>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10">
         <v>1</v>
       </c>
       <c r="W11" s="7">
@@ -2439,24 +2460,24 @@
       <c r="N12" s="7">
         <v>0</v>
       </c>
-      <c r="O12" s="8">
-        <v>0</v>
-      </c>
-      <c r="P12" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8">
-        <v>0</v>
-      </c>
-      <c r="S12" s="9">
-        <v>0</v>
-      </c>
-      <c r="T12" s="9">
-        <v>1</v>
-      </c>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9">
+      <c r="O12" s="9">
+        <v>0</v>
+      </c>
+      <c r="P12" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9">
+        <v>0</v>
+      </c>
+      <c r="S12" s="10">
+        <v>0</v>
+      </c>
+      <c r="T12" s="10">
+        <v>1</v>
+      </c>
+      <c r="U12" s="10"/>
+      <c r="V12" s="10">
         <v>0</v>
       </c>
       <c r="W12" s="7">
@@ -2507,24 +2528,24 @@
       <c r="N13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9" t="s">
+      <c r="O13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U13" s="10"/>
+      <c r="V13" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W13" s="7" t="s">
@@ -2575,24 +2596,24 @@
       <c r="N14" s="7">
         <v>0</v>
       </c>
-      <c r="O14" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P14" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S14" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T14" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9" t="s">
+      <c r="O14" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P14" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W14" s="7" t="s">
@@ -2643,24 +2664,24 @@
       <c r="N15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O15" s="8">
-        <v>0</v>
-      </c>
-      <c r="P15" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="8">
-        <v>1</v>
-      </c>
-      <c r="S15" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T15" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9" t="s">
+      <c r="O15" s="9">
+        <v>0</v>
+      </c>
+      <c r="P15" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9">
+        <v>1</v>
+      </c>
+      <c r="S15" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T15" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W15" s="7" t="s">
@@ -2711,24 +2732,24 @@
       <c r="N16" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S16" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T16" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9" t="s">
+      <c r="O16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S16" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T16" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U16" s="10"/>
+      <c r="V16" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W16" s="7">
@@ -2779,26 +2800,26 @@
       <c r="N17" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O17" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P17" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S17" s="9">
-        <v>1</v>
-      </c>
-      <c r="T17" s="9">
-        <v>1</v>
-      </c>
-      <c r="U17" s="9" t="s">
+      <c r="O17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S17" s="10">
+        <v>1</v>
+      </c>
+      <c r="T17" s="10">
+        <v>1</v>
+      </c>
+      <c r="U17" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="V17" s="9">
+      <c r="V17" s="10">
         <v>0</v>
       </c>
       <c r="W17" s="7" t="s">
@@ -2849,24 +2870,24 @@
       <c r="N18" s="7">
         <v>0</v>
       </c>
-      <c r="O18" s="8">
-        <v>0</v>
-      </c>
-      <c r="P18" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="8">
-        <v>0</v>
-      </c>
-      <c r="S18" s="9">
-        <v>0</v>
-      </c>
-      <c r="T18" s="9">
-        <v>1</v>
-      </c>
-      <c r="U18" s="9"/>
-      <c r="V18" s="9">
+      <c r="O18" s="9">
+        <v>0</v>
+      </c>
+      <c r="P18" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9">
+        <v>0</v>
+      </c>
+      <c r="S18" s="10">
+        <v>0</v>
+      </c>
+      <c r="T18" s="10">
+        <v>1</v>
+      </c>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10">
         <v>0</v>
       </c>
       <c r="W18" s="7">
@@ -2917,24 +2938,24 @@
       <c r="N19" s="7">
         <v>0</v>
       </c>
-      <c r="O19" s="8">
-        <v>1</v>
-      </c>
-      <c r="P19" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8">
-        <v>0</v>
-      </c>
-      <c r="S19" s="9">
-        <v>1</v>
-      </c>
-      <c r="T19" s="9">
-        <v>1</v>
-      </c>
-      <c r="U19" s="9"/>
-      <c r="V19" s="9">
+      <c r="O19" s="9">
+        <v>1</v>
+      </c>
+      <c r="P19" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9">
+        <v>0</v>
+      </c>
+      <c r="S19" s="10">
+        <v>1</v>
+      </c>
+      <c r="T19" s="10">
+        <v>1</v>
+      </c>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10">
         <v>0</v>
       </c>
       <c r="W19" s="7">
@@ -2985,24 +3006,24 @@
       <c r="N20" s="7">
         <v>0</v>
       </c>
-      <c r="O20" s="8">
-        <v>0</v>
-      </c>
-      <c r="P20" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8">
-        <v>0</v>
-      </c>
-      <c r="S20" s="9">
-        <v>0</v>
-      </c>
-      <c r="T20" s="9">
-        <v>1</v>
-      </c>
-      <c r="U20" s="9"/>
-      <c r="V20" s="9">
+      <c r="O20" s="9">
+        <v>0</v>
+      </c>
+      <c r="P20" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9">
+        <v>0</v>
+      </c>
+      <c r="S20" s="10">
+        <v>0</v>
+      </c>
+      <c r="T20" s="10">
+        <v>1</v>
+      </c>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10">
         <v>0</v>
       </c>
       <c r="W20" s="7">
@@ -3020,7 +3041,7 @@
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="2">
@@ -3053,24 +3074,24 @@
       <c r="N21" s="7">
         <v>1</v>
       </c>
-      <c r="O21" s="8">
-        <v>0</v>
-      </c>
-      <c r="P21" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="8"/>
-      <c r="R21" s="8">
-        <v>1</v>
-      </c>
-      <c r="S21" s="9">
-        <v>0</v>
-      </c>
-      <c r="T21" s="9">
-        <v>1</v>
-      </c>
-      <c r="U21" s="9"/>
-      <c r="V21" s="9">
+      <c r="O21" s="9">
+        <v>0</v>
+      </c>
+      <c r="P21" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9">
+        <v>1</v>
+      </c>
+      <c r="S21" s="10">
+        <v>0</v>
+      </c>
+      <c r="T21" s="10">
+        <v>1</v>
+      </c>
+      <c r="U21" s="10"/>
+      <c r="V21" s="10">
         <v>1</v>
       </c>
       <c r="W21" s="7" t="s">
@@ -3088,7 +3109,7 @@
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="17" t="s">
         <v>35</v>
       </c>
       <c r="C22" s="2">
@@ -3121,24 +3142,24 @@
       <c r="N22" s="7">
         <v>1</v>
       </c>
-      <c r="O22" s="8">
-        <v>1</v>
-      </c>
-      <c r="P22" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="8">
-        <v>1</v>
-      </c>
-      <c r="S22" s="9">
-        <v>1</v>
-      </c>
-      <c r="T22" s="9">
-        <v>1</v>
-      </c>
-      <c r="U22" s="9"/>
-      <c r="V22" s="9">
+      <c r="O22" s="9">
+        <v>1</v>
+      </c>
+      <c r="P22" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9">
+        <v>1</v>
+      </c>
+      <c r="S22" s="10">
+        <v>1</v>
+      </c>
+      <c r="T22" s="10">
+        <v>1</v>
+      </c>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10">
         <v>1</v>
       </c>
       <c r="W22" s="7" t="s">
@@ -3156,7 +3177,7 @@
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="17" t="s">
         <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -3189,24 +3210,24 @@
       <c r="N23" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O23" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P23" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q23" s="8"/>
-      <c r="R23" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S23" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T23" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U23" s="9"/>
-      <c r="V23" s="9" t="s">
+      <c r="O23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W23" s="7">
@@ -3222,7 +3243,7 @@
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="17" t="s">
         <v>37</v>
       </c>
       <c r="C24" s="2">
@@ -3255,24 +3276,24 @@
       <c r="N24" s="7">
         <v>1</v>
       </c>
-      <c r="O24" s="8">
-        <v>0</v>
-      </c>
-      <c r="P24" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="8">
-        <v>1</v>
-      </c>
-      <c r="S24" s="9">
-        <v>0</v>
-      </c>
-      <c r="T24" s="9">
-        <v>0</v>
-      </c>
-      <c r="U24" s="9"/>
-      <c r="V24" s="9">
+      <c r="O24" s="9">
+        <v>0</v>
+      </c>
+      <c r="P24" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9">
+        <v>1</v>
+      </c>
+      <c r="S24" s="10">
+        <v>0</v>
+      </c>
+      <c r="T24" s="10">
+        <v>0</v>
+      </c>
+      <c r="U24" s="10"/>
+      <c r="V24" s="10">
         <v>1</v>
       </c>
       <c r="W24" s="7">
@@ -3323,24 +3344,24 @@
       <c r="N25" s="7">
         <v>0</v>
       </c>
-      <c r="O25" s="8">
-        <v>0</v>
-      </c>
-      <c r="P25" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="8"/>
-      <c r="R25" s="8">
-        <v>0</v>
-      </c>
-      <c r="S25" s="9">
-        <v>0</v>
-      </c>
-      <c r="T25" s="9">
-        <v>1</v>
-      </c>
-      <c r="U25" s="9"/>
-      <c r="V25" s="9">
+      <c r="O25" s="9">
+        <v>0</v>
+      </c>
+      <c r="P25" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9">
+        <v>0</v>
+      </c>
+      <c r="S25" s="10">
+        <v>0</v>
+      </c>
+      <c r="T25" s="10">
+        <v>1</v>
+      </c>
+      <c r="U25" s="10"/>
+      <c r="V25" s="10">
         <v>0</v>
       </c>
       <c r="W25" s="7">
@@ -3391,24 +3412,24 @@
       <c r="N26" s="7">
         <v>0</v>
       </c>
-      <c r="O26" s="8">
-        <v>1</v>
-      </c>
-      <c r="P26" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="8">
-        <v>0</v>
-      </c>
-      <c r="S26" s="9">
-        <v>1</v>
-      </c>
-      <c r="T26" s="9">
-        <v>1</v>
-      </c>
-      <c r="U26" s="9"/>
-      <c r="V26" s="9">
+      <c r="O26" s="9">
+        <v>1</v>
+      </c>
+      <c r="P26" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9">
+        <v>0</v>
+      </c>
+      <c r="S26" s="10">
+        <v>1</v>
+      </c>
+      <c r="T26" s="10">
+        <v>1</v>
+      </c>
+      <c r="U26" s="10"/>
+      <c r="V26" s="10">
         <v>0</v>
       </c>
       <c r="W26" s="7">
@@ -3459,24 +3480,24 @@
       <c r="N27" s="7">
         <v>1</v>
       </c>
-      <c r="O27" s="8">
-        <v>1</v>
-      </c>
-      <c r="P27" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q27" s="8"/>
-      <c r="R27" s="8">
-        <v>1</v>
-      </c>
-      <c r="S27" s="9">
-        <v>1</v>
-      </c>
-      <c r="T27" s="9">
-        <v>1</v>
-      </c>
-      <c r="U27" s="9"/>
-      <c r="V27" s="9">
+      <c r="O27" s="9">
+        <v>1</v>
+      </c>
+      <c r="P27" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="9"/>
+      <c r="R27" s="9">
+        <v>1</v>
+      </c>
+      <c r="S27" s="10">
+        <v>1</v>
+      </c>
+      <c r="T27" s="10">
+        <v>1</v>
+      </c>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10">
         <v>1</v>
       </c>
       <c r="W27" s="7">
@@ -3527,24 +3548,24 @@
       <c r="N28" s="7">
         <v>1</v>
       </c>
-      <c r="O28" s="8">
-        <v>0</v>
-      </c>
-      <c r="P28" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q28" s="8"/>
-      <c r="R28" s="8">
-        <v>1</v>
-      </c>
-      <c r="S28" s="9">
-        <v>0</v>
-      </c>
-      <c r="T28" s="9">
-        <v>1</v>
-      </c>
-      <c r="U28" s="9"/>
-      <c r="V28" s="9">
+      <c r="O28" s="9">
+        <v>0</v>
+      </c>
+      <c r="P28" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="9"/>
+      <c r="R28" s="9">
+        <v>1</v>
+      </c>
+      <c r="S28" s="10">
+        <v>0</v>
+      </c>
+      <c r="T28" s="10">
+        <v>1</v>
+      </c>
+      <c r="U28" s="10"/>
+      <c r="V28" s="10">
         <v>1</v>
       </c>
       <c r="W28" s="7">
@@ -3595,24 +3616,24 @@
       <c r="N29" s="7">
         <v>0</v>
       </c>
-      <c r="O29" s="8">
-        <v>0</v>
-      </c>
-      <c r="P29" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q29" s="8"/>
-      <c r="R29" s="8">
-        <v>0</v>
-      </c>
-      <c r="S29" s="9">
-        <v>0</v>
-      </c>
-      <c r="T29" s="9">
-        <v>1</v>
-      </c>
-      <c r="U29" s="9"/>
-      <c r="V29" s="9">
+      <c r="O29" s="9">
+        <v>0</v>
+      </c>
+      <c r="P29" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9">
+        <v>0</v>
+      </c>
+      <c r="S29" s="10">
+        <v>0</v>
+      </c>
+      <c r="T29" s="10">
+        <v>1</v>
+      </c>
+      <c r="U29" s="10"/>
+      <c r="V29" s="10">
         <v>0</v>
       </c>
       <c r="W29" s="7">
@@ -3663,24 +3684,24 @@
       <c r="N30" s="7">
         <v>0</v>
       </c>
-      <c r="O30" s="8">
-        <v>0</v>
-      </c>
-      <c r="P30" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="8">
-        <v>0</v>
-      </c>
-      <c r="S30" s="9">
-        <v>0</v>
-      </c>
-      <c r="T30" s="9">
-        <v>1</v>
-      </c>
-      <c r="U30" s="9"/>
-      <c r="V30" s="9">
+      <c r="O30" s="9">
+        <v>0</v>
+      </c>
+      <c r="P30" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9">
+        <v>0</v>
+      </c>
+      <c r="S30" s="10">
+        <v>0</v>
+      </c>
+      <c r="T30" s="10">
+        <v>1</v>
+      </c>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10">
         <v>0</v>
       </c>
       <c r="W30" s="7">
@@ -3731,24 +3752,24 @@
       <c r="N31" s="7">
         <v>0</v>
       </c>
-      <c r="O31" s="8">
-        <v>0</v>
-      </c>
-      <c r="P31" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="8"/>
-      <c r="R31" s="8">
-        <v>0</v>
-      </c>
-      <c r="S31" s="9">
-        <v>0</v>
-      </c>
-      <c r="T31" s="9">
-        <v>1</v>
-      </c>
-      <c r="U31" s="9"/>
-      <c r="V31" s="9">
+      <c r="O31" s="9">
+        <v>0</v>
+      </c>
+      <c r="P31" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9">
+        <v>0</v>
+      </c>
+      <c r="S31" s="10">
+        <v>0</v>
+      </c>
+      <c r="T31" s="10">
+        <v>1</v>
+      </c>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10">
         <v>0</v>
       </c>
       <c r="W31" s="7">
@@ -3799,24 +3820,24 @@
       <c r="N32" s="7">
         <v>0</v>
       </c>
-      <c r="O32" s="8">
-        <v>0</v>
-      </c>
-      <c r="P32" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q32" s="8"/>
-      <c r="R32" s="8">
-        <v>0</v>
-      </c>
-      <c r="S32" s="9">
-        <v>0</v>
-      </c>
-      <c r="T32" s="9">
-        <v>1</v>
-      </c>
-      <c r="U32" s="9"/>
-      <c r="V32" s="9">
+      <c r="O32" s="9">
+        <v>0</v>
+      </c>
+      <c r="P32" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9">
+        <v>0</v>
+      </c>
+      <c r="S32" s="10">
+        <v>0</v>
+      </c>
+      <c r="T32" s="10">
+        <v>1</v>
+      </c>
+      <c r="U32" s="10"/>
+      <c r="V32" s="10">
         <v>0</v>
       </c>
       <c r="W32" s="7">
@@ -3899,28 +3920,28 @@
       <c r="N1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="10" t="s">
         <v>5</v>
       </c>
       <c r="W1" s="7" t="s">
@@ -3979,28 +4000,28 @@
       <c r="N2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="P2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="R2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="T2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="V2" s="9" t="s">
+      <c r="V2" s="10" t="s">
         <v>12</v>
       </c>
       <c r="W2" s="7" t="s">
@@ -4053,24 +4074,24 @@
       <c r="N3" s="7">
         <v>1</v>
       </c>
-      <c r="O3" s="8">
-        <v>1</v>
-      </c>
-      <c r="P3" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8">
-        <v>1</v>
-      </c>
-      <c r="S3" s="9">
-        <v>1</v>
-      </c>
-      <c r="T3" s="9">
-        <v>1</v>
-      </c>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9">
+      <c r="O3" s="9">
+        <v>1</v>
+      </c>
+      <c r="P3" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9">
+        <v>1</v>
+      </c>
+      <c r="S3" s="10">
+        <v>1</v>
+      </c>
+      <c r="T3" s="10">
+        <v>1</v>
+      </c>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10">
         <v>1</v>
       </c>
       <c r="W3" s="7">
@@ -4121,24 +4142,24 @@
       <c r="N4" s="7">
         <v>0</v>
       </c>
-      <c r="O4" s="8">
-        <v>0</v>
-      </c>
-      <c r="P4" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8">
-        <v>0</v>
-      </c>
-      <c r="S4" s="9">
-        <v>0</v>
-      </c>
-      <c r="T4" s="9">
-        <v>1</v>
-      </c>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9">
+      <c r="O4" s="9">
+        <v>0</v>
+      </c>
+      <c r="P4" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9">
+        <v>0</v>
+      </c>
+      <c r="S4" s="10">
+        <v>0</v>
+      </c>
+      <c r="T4" s="10">
+        <v>1</v>
+      </c>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10">
         <v>0</v>
       </c>
       <c r="W4" s="7">
@@ -4189,24 +4210,24 @@
       <c r="N5" s="7">
         <v>1</v>
       </c>
-      <c r="O5" s="8">
-        <v>1</v>
-      </c>
-      <c r="P5" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8">
-        <v>1</v>
-      </c>
-      <c r="S5" s="9">
-        <v>1</v>
-      </c>
-      <c r="T5" s="9">
-        <v>1</v>
-      </c>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9">
+      <c r="O5" s="9">
+        <v>1</v>
+      </c>
+      <c r="P5" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9">
+        <v>1</v>
+      </c>
+      <c r="S5" s="10">
+        <v>1</v>
+      </c>
+      <c r="T5" s="10">
+        <v>1</v>
+      </c>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10">
         <v>1</v>
       </c>
       <c r="W5" s="7" t="s">
@@ -4257,24 +4278,24 @@
       <c r="N6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T6" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9" t="s">
+      <c r="O6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W6" s="7">
@@ -4327,24 +4348,24 @@
       <c r="N7" s="7">
         <v>0</v>
       </c>
-      <c r="O7" s="8">
-        <v>1</v>
-      </c>
-      <c r="P7" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8">
-        <v>0</v>
-      </c>
-      <c r="S7" s="9">
-        <v>1</v>
-      </c>
-      <c r="T7" s="9">
-        <v>1</v>
-      </c>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9">
+      <c r="O7" s="9">
+        <v>1</v>
+      </c>
+      <c r="P7" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9">
+        <v>0</v>
+      </c>
+      <c r="S7" s="10">
+        <v>1</v>
+      </c>
+      <c r="T7" s="10">
+        <v>1</v>
+      </c>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10">
         <v>0</v>
       </c>
       <c r="W7" s="7" t="s">
@@ -4397,26 +4418,26 @@
       <c r="N8" s="7">
         <v>1</v>
       </c>
-      <c r="O8" s="8">
-        <v>1</v>
-      </c>
-      <c r="P8" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8">
-        <v>1</v>
-      </c>
-      <c r="S8" s="9">
-        <v>1</v>
-      </c>
-      <c r="T8" s="9">
-        <v>1</v>
-      </c>
-      <c r="U8" s="9" t="s">
+      <c r="O8" s="9">
+        <v>1</v>
+      </c>
+      <c r="P8" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9">
+        <v>1</v>
+      </c>
+      <c r="S8" s="10">
+        <v>1</v>
+      </c>
+      <c r="T8" s="10">
+        <v>1</v>
+      </c>
+      <c r="U8" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="V8" s="9">
+      <c r="V8" s="10">
         <v>1</v>
       </c>
       <c r="W8" s="7" t="s">
@@ -4469,28 +4490,28 @@
       <c r="N9" s="7">
         <v>1</v>
       </c>
-      <c r="O9" s="8">
-        <v>1</v>
-      </c>
-      <c r="P9" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="8" t="s">
+      <c r="O9" s="9">
+        <v>1</v>
+      </c>
+      <c r="P9" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="R9" s="8">
-        <v>1</v>
-      </c>
-      <c r="S9" s="9">
-        <v>1</v>
-      </c>
-      <c r="T9" s="9">
-        <v>1</v>
-      </c>
-      <c r="U9" s="9" t="s">
+      <c r="R9" s="9">
+        <v>1</v>
+      </c>
+      <c r="S9" s="10">
+        <v>1</v>
+      </c>
+      <c r="T9" s="10">
+        <v>1</v>
+      </c>
+      <c r="U9" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="V9" s="9">
+      <c r="V9" s="10">
         <v>1</v>
       </c>
       <c r="W9" s="7" t="s">
@@ -4543,28 +4564,28 @@
       <c r="N10" s="7">
         <v>1</v>
       </c>
-      <c r="O10" s="8">
-        <v>1</v>
-      </c>
-      <c r="P10" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="8" t="s">
+      <c r="O10" s="9">
+        <v>1</v>
+      </c>
+      <c r="P10" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="R10" s="8">
-        <v>1</v>
-      </c>
-      <c r="S10" s="9">
-        <v>1</v>
-      </c>
-      <c r="T10" s="9">
-        <v>1</v>
-      </c>
-      <c r="U10" s="9" t="s">
+      <c r="R10" s="9">
+        <v>1</v>
+      </c>
+      <c r="S10" s="10">
+        <v>1</v>
+      </c>
+      <c r="T10" s="10">
+        <v>1</v>
+      </c>
+      <c r="U10" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="V10" s="9">
+      <c r="V10" s="10">
         <v>0</v>
       </c>
       <c r="W10" s="7">
@@ -4619,26 +4640,26 @@
       <c r="N11" s="7">
         <v>0</v>
       </c>
-      <c r="O11" s="8">
-        <v>1</v>
-      </c>
-      <c r="P11" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="8" t="s">
+      <c r="O11" s="9">
+        <v>1</v>
+      </c>
+      <c r="P11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="R11" s="8">
-        <v>0</v>
-      </c>
-      <c r="S11" s="9">
-        <v>1</v>
-      </c>
-      <c r="T11" s="9">
-        <v>1</v>
-      </c>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9">
+      <c r="R11" s="9">
+        <v>0</v>
+      </c>
+      <c r="S11" s="10">
+        <v>1</v>
+      </c>
+      <c r="T11" s="10">
+        <v>1</v>
+      </c>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10">
         <v>0</v>
       </c>
       <c r="W11" s="7">
@@ -4689,24 +4710,24 @@
       <c r="N12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S12" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T12" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9" t="s">
+      <c r="O12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S12" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T12" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U12" s="10"/>
+      <c r="V12" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W12" s="7">
@@ -4759,24 +4780,24 @@
       <c r="N13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9" t="s">
+      <c r="O13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U13" s="10"/>
+      <c r="V13" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W13" s="7">
@@ -4831,26 +4852,26 @@
       <c r="N14" s="7">
         <v>0</v>
       </c>
-      <c r="O14" s="8">
-        <v>1</v>
-      </c>
-      <c r="P14" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="8" t="s">
+      <c r="O14" s="9">
+        <v>1</v>
+      </c>
+      <c r="P14" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="R14" s="8">
-        <v>0</v>
-      </c>
-      <c r="S14" s="9">
-        <v>1</v>
-      </c>
-      <c r="T14" s="9">
-        <v>1</v>
-      </c>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9">
+      <c r="R14" s="9">
+        <v>0</v>
+      </c>
+      <c r="S14" s="10">
+        <v>1</v>
+      </c>
+      <c r="T14" s="10">
+        <v>1</v>
+      </c>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10">
         <v>0</v>
       </c>
       <c r="W14" s="7">
@@ -4903,24 +4924,24 @@
       <c r="N15" s="7">
         <v>1</v>
       </c>
-      <c r="O15" s="8">
-        <v>1</v>
-      </c>
-      <c r="P15" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="8">
-        <v>1</v>
-      </c>
-      <c r="S15" s="9">
-        <v>1</v>
-      </c>
-      <c r="T15" s="9">
-        <v>1</v>
-      </c>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9">
+      <c r="O15" s="9">
+        <v>1</v>
+      </c>
+      <c r="P15" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9">
+        <v>1</v>
+      </c>
+      <c r="S15" s="10">
+        <v>1</v>
+      </c>
+      <c r="T15" s="10">
+        <v>1</v>
+      </c>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10">
         <v>1</v>
       </c>
       <c r="W15" s="7" t="s">
@@ -4971,24 +4992,24 @@
       <c r="N16" s="7">
         <v>0</v>
       </c>
-      <c r="O16" s="8">
-        <v>1</v>
-      </c>
-      <c r="P16" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="8">
-        <v>0</v>
-      </c>
-      <c r="S16" s="9">
-        <v>1</v>
-      </c>
-      <c r="T16" s="9">
-        <v>1</v>
-      </c>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9">
+      <c r="O16" s="9">
+        <v>1</v>
+      </c>
+      <c r="P16" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9">
+        <v>0</v>
+      </c>
+      <c r="S16" s="10">
+        <v>1</v>
+      </c>
+      <c r="T16" s="10">
+        <v>1</v>
+      </c>
+      <c r="U16" s="10"/>
+      <c r="V16" s="10">
         <v>0</v>
       </c>
       <c r="W16" s="7" t="s">
@@ -5041,24 +5062,24 @@
       <c r="N17" s="7">
         <v>1</v>
       </c>
-      <c r="O17" s="8">
-        <v>1</v>
-      </c>
-      <c r="P17" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="8"/>
-      <c r="R17" s="8">
-        <v>1</v>
-      </c>
-      <c r="S17" s="9">
-        <v>1</v>
-      </c>
-      <c r="T17" s="9">
-        <v>1</v>
-      </c>
-      <c r="U17" s="9"/>
-      <c r="V17" s="9">
+      <c r="O17" s="9">
+        <v>1</v>
+      </c>
+      <c r="P17" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9">
+        <v>1</v>
+      </c>
+      <c r="S17" s="10">
+        <v>1</v>
+      </c>
+      <c r="T17" s="10">
+        <v>1</v>
+      </c>
+      <c r="U17" s="10"/>
+      <c r="V17" s="10">
         <v>1</v>
       </c>
       <c r="W17" s="7">
@@ -5109,24 +5130,24 @@
       <c r="N18" s="7">
         <v>1</v>
       </c>
-      <c r="O18" s="8">
-        <v>1</v>
-      </c>
-      <c r="P18" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="8"/>
-      <c r="R18" s="8">
-        <v>1</v>
-      </c>
-      <c r="S18" s="9">
-        <v>1</v>
-      </c>
-      <c r="T18" s="9">
-        <v>1</v>
-      </c>
-      <c r="U18" s="9"/>
-      <c r="V18" s="9">
+      <c r="O18" s="9">
+        <v>1</v>
+      </c>
+      <c r="P18" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9">
+        <v>1</v>
+      </c>
+      <c r="S18" s="10">
+        <v>1</v>
+      </c>
+      <c r="T18" s="10">
+        <v>1</v>
+      </c>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10">
         <v>1</v>
       </c>
       <c r="W18" s="7">
@@ -5177,24 +5198,24 @@
       <c r="N19" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O19" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P19" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S19" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T19" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U19" s="9"/>
-      <c r="V19" s="9" t="s">
+      <c r="O19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S19" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T19" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W19" s="7">
@@ -5245,24 +5266,24 @@
       <c r="N20" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O20" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P20" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S20" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T20" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U20" s="9"/>
-      <c r="V20" s="9" t="s">
+      <c r="O20" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P20" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S20" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T20" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W20" s="7">
@@ -5280,7 +5301,7 @@
       <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="14" t="s">
         <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -5313,24 +5334,24 @@
       <c r="N21" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O21" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P21" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q21" s="8"/>
-      <c r="R21" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S21" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T21" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U21" s="9"/>
-      <c r="V21" s="9" t="s">
+      <c r="O21" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P21" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S21" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T21" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U21" s="10"/>
+      <c r="V21" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W21" s="7">
@@ -5381,24 +5402,24 @@
       <c r="N22" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O22" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P22" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S22" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T22" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U22" s="9"/>
-      <c r="V22" s="9" t="s">
+      <c r="O22" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P22" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S22" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T22" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W22" s="7">
@@ -5449,24 +5470,24 @@
       <c r="N23" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O23" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P23" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q23" s="8"/>
-      <c r="R23" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S23" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T23" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U23" s="9"/>
-      <c r="V23" s="9" t="s">
+      <c r="O23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W23" s="7">
@@ -5517,24 +5538,24 @@
       <c r="N24" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O24" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P24" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S24" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T24" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U24" s="9"/>
-      <c r="V24" s="9" t="s">
+      <c r="O24" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P24" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S24" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T24" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U24" s="10"/>
+      <c r="V24" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W24" s="7">
@@ -5587,24 +5608,24 @@
       <c r="N25" s="7">
         <v>1</v>
       </c>
-      <c r="O25" s="8">
-        <v>1</v>
-      </c>
-      <c r="P25" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="8"/>
-      <c r="R25" s="8">
-        <v>1</v>
-      </c>
-      <c r="S25" s="9">
-        <v>1</v>
-      </c>
-      <c r="T25" s="9">
-        <v>1</v>
-      </c>
-      <c r="U25" s="9"/>
-      <c r="V25" s="9">
+      <c r="O25" s="9">
+        <v>1</v>
+      </c>
+      <c r="P25" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9">
+        <v>1</v>
+      </c>
+      <c r="S25" s="10">
+        <v>1</v>
+      </c>
+      <c r="T25" s="10">
+        <v>1</v>
+      </c>
+      <c r="U25" s="10"/>
+      <c r="V25" s="10">
         <v>1</v>
       </c>
       <c r="W25" s="7" t="s">
@@ -5655,24 +5676,24 @@
       <c r="N26" s="7">
         <v>1</v>
       </c>
-      <c r="O26" s="8">
-        <v>1</v>
-      </c>
-      <c r="P26" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="8">
-        <v>1</v>
-      </c>
-      <c r="S26" s="9">
-        <v>1</v>
-      </c>
-      <c r="T26" s="9">
-        <v>0</v>
-      </c>
-      <c r="U26" s="9"/>
-      <c r="V26" s="9">
+      <c r="O26" s="9">
+        <v>1</v>
+      </c>
+      <c r="P26" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9">
+        <v>1</v>
+      </c>
+      <c r="S26" s="10">
+        <v>1</v>
+      </c>
+      <c r="T26" s="10">
+        <v>0</v>
+      </c>
+      <c r="U26" s="10"/>
+      <c r="V26" s="10">
         <v>1</v>
       </c>
       <c r="W26" s="7">
@@ -5725,24 +5746,24 @@
       <c r="N27" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O27" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P27" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q27" s="8"/>
-      <c r="R27" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S27" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T27" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U27" s="9"/>
-      <c r="V27" s="9" t="s">
+      <c r="O27" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P27" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q27" s="9"/>
+      <c r="R27" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S27" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T27" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W27" s="7" t="s">
@@ -5793,24 +5814,24 @@
       <c r="N28" s="7">
         <v>1</v>
       </c>
-      <c r="O28" s="8">
-        <v>1</v>
-      </c>
-      <c r="P28" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q28" s="8"/>
-      <c r="R28" s="8">
-        <v>1</v>
-      </c>
-      <c r="S28" s="9">
-        <v>1</v>
-      </c>
-      <c r="T28" s="9">
-        <v>1</v>
-      </c>
-      <c r="U28" s="9"/>
-      <c r="V28" s="9">
+      <c r="O28" s="9">
+        <v>1</v>
+      </c>
+      <c r="P28" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="9"/>
+      <c r="R28" s="9">
+        <v>1</v>
+      </c>
+      <c r="S28" s="10">
+        <v>1</v>
+      </c>
+      <c r="T28" s="10">
+        <v>1</v>
+      </c>
+      <c r="U28" s="10"/>
+      <c r="V28" s="10">
         <v>1</v>
       </c>
       <c r="W28" s="7">
@@ -5861,24 +5882,24 @@
       <c r="N29" s="7">
         <v>1</v>
       </c>
-      <c r="O29" s="8">
-        <v>1</v>
-      </c>
-      <c r="P29" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="8"/>
-      <c r="R29" s="8">
-        <v>1</v>
-      </c>
-      <c r="S29" s="9">
-        <v>1</v>
-      </c>
-      <c r="T29" s="9">
-        <v>0</v>
-      </c>
-      <c r="U29" s="9"/>
-      <c r="V29" s="9">
+      <c r="O29" s="9">
+        <v>1</v>
+      </c>
+      <c r="P29" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9">
+        <v>1</v>
+      </c>
+      <c r="S29" s="10">
+        <v>1</v>
+      </c>
+      <c r="T29" s="10">
+        <v>0</v>
+      </c>
+      <c r="U29" s="10"/>
+      <c r="V29" s="10">
         <v>1</v>
       </c>
       <c r="W29" s="7" t="s">
@@ -5927,24 +5948,24 @@
       <c r="N30" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S30" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="T30" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="U30" s="9"/>
-      <c r="V30" s="9" t="s">
+      <c r="O30" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P30" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="S30" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T30" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10" t="s">
         <v>20</v>
       </c>
       <c r="W30" s="7">
@@ -5995,24 +6016,24 @@
       <c r="N31" s="7">
         <v>1</v>
       </c>
-      <c r="O31" s="8">
-        <v>1</v>
-      </c>
-      <c r="P31" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="8"/>
-      <c r="R31" s="8">
-        <v>1</v>
-      </c>
-      <c r="S31" s="9">
-        <v>1</v>
-      </c>
-      <c r="T31" s="9">
-        <v>1</v>
-      </c>
-      <c r="U31" s="9"/>
-      <c r="V31" s="9">
+      <c r="O31" s="9">
+        <v>1</v>
+      </c>
+      <c r="P31" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9">
+        <v>1</v>
+      </c>
+      <c r="S31" s="10">
+        <v>1</v>
+      </c>
+      <c r="T31" s="10">
+        <v>1</v>
+      </c>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10">
         <v>1</v>
       </c>
       <c r="W31" s="7">
@@ -6063,24 +6084,24 @@
       <c r="N32" s="7">
         <v>1</v>
       </c>
-      <c r="O32" s="8">
-        <v>1</v>
-      </c>
-      <c r="P32" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q32" s="8"/>
-      <c r="R32" s="8">
-        <v>1</v>
-      </c>
-      <c r="S32" s="9">
-        <v>1</v>
-      </c>
-      <c r="T32" s="9">
-        <v>1</v>
-      </c>
-      <c r="U32" s="9"/>
-      <c r="V32" s="9">
+      <c r="O32" s="9">
+        <v>1</v>
+      </c>
+      <c r="P32" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9">
+        <v>1</v>
+      </c>
+      <c r="S32" s="10">
+        <v>1</v>
+      </c>
+      <c r="T32" s="10">
+        <v>1</v>
+      </c>
+      <c r="U32" s="10"/>
+      <c r="V32" s="10">
         <v>1</v>
       </c>
       <c r="W32" s="7">
@@ -6131,24 +6152,24 @@
       <c r="N33" s="7">
         <v>1</v>
       </c>
-      <c r="O33" s="8">
-        <v>1</v>
-      </c>
-      <c r="P33" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q33" s="8"/>
-      <c r="R33" s="8">
-        <v>1</v>
-      </c>
-      <c r="S33" s="9">
-        <v>1</v>
-      </c>
-      <c r="T33" s="9">
-        <v>1</v>
-      </c>
-      <c r="U33" s="9"/>
-      <c r="V33" s="9">
+      <c r="O33" s="9">
+        <v>1</v>
+      </c>
+      <c r="P33" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9">
+        <v>1</v>
+      </c>
+      <c r="S33" s="10">
+        <v>1</v>
+      </c>
+      <c r="T33" s="10">
+        <v>1</v>
+      </c>
+      <c r="U33" s="10"/>
+      <c r="V33" s="10">
         <v>1</v>
       </c>
       <c r="W33" s="7">
@@ -6199,24 +6220,24 @@
       <c r="N34" s="7">
         <v>1</v>
       </c>
-      <c r="O34" s="8">
-        <v>0</v>
-      </c>
-      <c r="P34" s="8">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="8"/>
-      <c r="R34" s="8">
-        <v>1</v>
-      </c>
-      <c r="S34" s="9">
-        <v>0</v>
-      </c>
-      <c r="T34" s="9">
-        <v>0</v>
-      </c>
-      <c r="U34" s="9"/>
-      <c r="V34" s="9">
+      <c r="O34" s="9">
+        <v>0</v>
+      </c>
+      <c r="P34" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9">
+        <v>1</v>
+      </c>
+      <c r="S34" s="10">
+        <v>0</v>
+      </c>
+      <c r="T34" s="10">
+        <v>0</v>
+      </c>
+      <c r="U34" s="10"/>
+      <c r="V34" s="10">
         <v>1</v>
       </c>
       <c r="W34" s="7">
@@ -6267,24 +6288,24 @@
       <c r="N35" s="7">
         <v>0</v>
       </c>
-      <c r="O35" s="8">
-        <v>0</v>
-      </c>
-      <c r="P35" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="8"/>
-      <c r="R35" s="8">
-        <v>0</v>
-      </c>
-      <c r="S35" s="9">
-        <v>0</v>
-      </c>
-      <c r="T35" s="9">
-        <v>1</v>
-      </c>
-      <c r="U35" s="9"/>
-      <c r="V35" s="9">
+      <c r="O35" s="9">
+        <v>0</v>
+      </c>
+      <c r="P35" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9">
+        <v>0</v>
+      </c>
+      <c r="S35" s="10">
+        <v>0</v>
+      </c>
+      <c r="T35" s="10">
+        <v>1</v>
+      </c>
+      <c r="U35" s="10"/>
+      <c r="V35" s="10">
         <v>0</v>
       </c>
       <c r="W35" s="7">
@@ -6302,7 +6323,7 @@
       <c r="A36" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="14" t="s">
         <v>100</v>
       </c>
       <c r="C36" s="2">
@@ -6335,24 +6356,24 @@
       <c r="N36" s="7">
         <v>1</v>
       </c>
-      <c r="O36" s="8">
-        <v>1</v>
-      </c>
-      <c r="P36" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8">
-        <v>1</v>
-      </c>
-      <c r="S36" s="9">
-        <v>1</v>
-      </c>
-      <c r="T36" s="9">
-        <v>1</v>
-      </c>
-      <c r="U36" s="9"/>
-      <c r="V36" s="9">
+      <c r="O36" s="9">
+        <v>1</v>
+      </c>
+      <c r="P36" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9">
+        <v>1</v>
+      </c>
+      <c r="S36" s="10">
+        <v>1</v>
+      </c>
+      <c r="T36" s="10">
+        <v>1</v>
+      </c>
+      <c r="U36" s="10"/>
+      <c r="V36" s="10">
         <v>1</v>
       </c>
       <c r="W36" s="7">
@@ -6375,10 +6396,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6"/>
+  <cols>
+    <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
+    <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
+    <col min="11" max="18" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:30">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6408,55 +6434,67 @@
         <v>2</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="O1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="S1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="T1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="U1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="V1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="W1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="X1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="Y1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="Z1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="AB1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="AC1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AD1" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:30">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -6484,10 +6522,10 @@
       <c r="I2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="11" t="s">
         <v>9</v>
       </c>
       <c r="L2" s="7" t="s">
@@ -6523,25 +6561,37 @@
       <c r="V2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="W2" s="7" t="s">
+      <c r="W2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="X2" s="7" t="s">
+      <c r="X2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="Y2" s="7" t="s">
+      <c r="Y2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="Z2" s="7" t="s">
+      <c r="Z2" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:26">
+      <c r="AA2" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD2" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30">
       <c r="A3" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>20</v>
@@ -6560,52 +6610,68 @@
         <v>1</v>
       </c>
       <c r="I3" s="5"/>
-      <c r="J3" s="6">
-        <v>0</v>
-      </c>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
+      <c r="J3" s="5">
+        <v>0</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>20</v>
+      <c r="N3" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="8">
+        <v>1</v>
+      </c>
+      <c r="P3" s="8">
+        <v>1</v>
       </c>
       <c r="Q3" s="8"/>
-      <c r="R3" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S3" s="9">
-        <v>1</v>
-      </c>
-      <c r="T3" s="9">
-        <v>1</v>
-      </c>
-      <c r="U3" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="V3" s="9">
-        <v>0</v>
-      </c>
-      <c r="W3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="X3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y3" s="7"/>
-      <c r="Z3" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26">
+      <c r="R3" s="13">
+        <v>0</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="W3" s="10">
+        <v>1</v>
+      </c>
+      <c r="X3" s="10">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z3" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC3" s="7"/>
+      <c r="AD3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30">
       <c r="A4" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -6624,50 +6690,66 @@
         <v>1</v>
       </c>
       <c r="I4" s="5"/>
-      <c r="J4" s="6">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
+      <c r="J4" s="5">
+        <v>0</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P4" s="8" t="s">
-        <v>20</v>
+      <c r="N4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="O4" s="8">
+        <v>0</v>
+      </c>
+      <c r="P4" s="8">
+        <v>1</v>
       </c>
       <c r="Q4" s="8"/>
-      <c r="R4" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S4" s="9">
-        <v>1</v>
-      </c>
-      <c r="T4" s="9">
-        <v>1</v>
+      <c r="R4" s="13">
+        <v>0</v>
+      </c>
+      <c r="S4" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="T4" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="U4" s="9"/>
-      <c r="V4" s="9">
-        <v>0</v>
-      </c>
-      <c r="W4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="X4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y4" s="7"/>
-      <c r="Z4" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26">
+      <c r="V4" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="W4" s="10">
+        <v>1</v>
+      </c>
+      <c r="X4" s="10">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="10"/>
+      <c r="Z4" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC4" s="7"/>
+      <c r="AD4" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30">
       <c r="A5" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>20</v>
@@ -6686,50 +6768,66 @@
         <v>1</v>
       </c>
       <c r="I5" s="5"/>
-      <c r="J5" s="6">
-        <v>0</v>
-      </c>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
+      <c r="J5" s="5">
+        <v>0</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P5" s="8" t="s">
-        <v>20</v>
+      <c r="N5" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="O5" s="8">
+        <v>0</v>
+      </c>
+      <c r="P5" s="8">
+        <v>1</v>
       </c>
       <c r="Q5" s="8"/>
-      <c r="R5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S5" s="9">
-        <v>1</v>
-      </c>
-      <c r="T5" s="9">
-        <v>1</v>
+      <c r="R5" s="13">
+        <v>0</v>
+      </c>
+      <c r="S5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="U5" s="9"/>
-      <c r="V5" s="9">
-        <v>0</v>
-      </c>
-      <c r="W5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="X5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y5" s="7"/>
-      <c r="Z5" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26">
+      <c r="V5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="W5" s="10">
+        <v>1</v>
+      </c>
+      <c r="X5" s="10">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="10"/>
+      <c r="Z5" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC5" s="7"/>
+      <c r="AD5" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30">
       <c r="A6" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -6748,47 +6846,63 @@
         <v>1</v>
       </c>
       <c r="I6" s="5"/>
-      <c r="J6" s="6">
-        <v>0</v>
-      </c>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
+      <c r="J6" s="5">
+        <v>0</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>20</v>
+      <c r="N6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="O6" s="8">
+        <v>0</v>
+      </c>
+      <c r="P6" s="8">
+        <v>1</v>
       </c>
       <c r="Q6" s="8"/>
-      <c r="R6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S6" s="9">
-        <v>1</v>
-      </c>
-      <c r="T6" s="9">
-        <v>1</v>
+      <c r="R6" s="13">
+        <v>0</v>
+      </c>
+      <c r="S6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="T6" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="U6" s="9"/>
-      <c r="V6" s="9">
-        <v>0</v>
-      </c>
-      <c r="W6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="X6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y6" s="7"/>
-      <c r="Z6" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26">
+      <c r="V6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="W6" s="10">
+        <v>1</v>
+      </c>
+      <c r="X6" s="10">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="10"/>
+      <c r="Z6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC6" s="7"/>
+      <c r="AD6" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30">
       <c r="A7" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>
@@ -6810,41 +6924,57 @@
         <v>1</v>
       </c>
       <c r="I7" s="5"/>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
+      <c r="J7" s="5">
+        <v>0</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P7" s="8" t="s">
-        <v>20</v>
+      <c r="N7" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="O7" s="8">
+        <v>0</v>
+      </c>
+      <c r="P7" s="8">
+        <v>1</v>
       </c>
       <c r="Q7" s="8"/>
-      <c r="R7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="S7" s="9">
-        <v>1</v>
-      </c>
-      <c r="T7" s="9">
-        <v>1</v>
+      <c r="R7" s="13">
+        <v>0</v>
+      </c>
+      <c r="S7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="T7" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="U7" s="9"/>
-      <c r="V7" s="9">
-        <v>0</v>
-      </c>
-      <c r="W7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="X7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y7" s="7"/>
-      <c r="Z7" s="7" t="s">
+      <c r="V7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="W7" s="10">
+        <v>1</v>
+      </c>
+      <c r="X7" s="10">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="10"/>
+      <c r="Z7" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC7" s="7"/>
+      <c r="AD7" s="7" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-06-11 11:15:33
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15020" activeTab="2"/>
+    <workbookView windowHeight="15020" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -6402,6 +6402,10 @@
     <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
     <col min="11" max="18" width="20" customWidth="1"/>
+    <col min="19" max="19" width="10.3076923076923" customWidth="1"/>
+    <col min="20" max="20" width="15.1538461538462" customWidth="1"/>
+    <col min="21" max="21" width="10.3076923076923" customWidth="1"/>
+    <col min="22" max="22" width="12.7692307692308" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30">

</xml_diff>

<commit_message>
vault backup: 2026-06-11 11:17:55
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15020" activeTab="1"/>
+    <workbookView windowHeight="15020" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="110">
   <si>
     <t>招标方式</t>
   </si>
@@ -336,6 +336,12 @@
   </si>
   <si>
     <t>询比采购（邀请）</t>
+  </si>
+  <si>
+    <t>谈判采购（公开）</t>
+  </si>
+  <si>
+    <t>谈判采购（邀请）</t>
   </si>
   <si>
     <t>邀请供应商</t>
@@ -519,7 +525,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -553,6 +559,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -922,7 +934,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -946,16 +958,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -964,89 +976,89 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1080,6 +1092,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1087,6 +1102,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1631,22 +1649,22 @@
   <cols>
     <col min="1" max="1" width="16.3846153846154" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="22.4615384615385" style="15" customWidth="1"/>
-    <col min="4" max="5" width="15.1538461538462" style="15" customWidth="1"/>
-    <col min="6" max="6" width="12.7692307692308" style="15" customWidth="1"/>
-    <col min="7" max="7" width="22.4615384615385" style="16" customWidth="1"/>
-    <col min="8" max="9" width="15.1538461538462" style="16" customWidth="1"/>
-    <col min="10" max="10" width="10.3076923076923" style="16" customWidth="1"/>
-    <col min="11" max="11" width="10.3076923076923" style="15" customWidth="1"/>
-    <col min="12" max="12" width="15.1538461538462" style="15" customWidth="1"/>
-    <col min="13" max="13" width="22.4615384615385" style="15" customWidth="1"/>
-    <col min="14" max="14" width="12.7692307692308" style="15" customWidth="1"/>
-    <col min="15" max="16" width="15.1538461538462" style="15" customWidth="1"/>
-    <col min="17" max="17" width="18.6923076923077" style="15" customWidth="1"/>
-    <col min="18" max="18" width="12.7692307692308" style="15" customWidth="1"/>
-    <col min="19" max="20" width="15.1538461538462" style="15" customWidth="1"/>
-    <col min="21" max="21" width="24.8461538461538" style="15" customWidth="1"/>
-    <col min="22" max="22" width="12.7692307692308" style="15" customWidth="1"/>
+    <col min="3" max="3" width="22.4615384615385" style="17" customWidth="1"/>
+    <col min="4" max="5" width="15.1538461538462" style="17" customWidth="1"/>
+    <col min="6" max="6" width="12.7692307692308" style="17" customWidth="1"/>
+    <col min="7" max="7" width="22.4615384615385" style="18" customWidth="1"/>
+    <col min="8" max="9" width="15.1538461538462" style="18" customWidth="1"/>
+    <col min="10" max="10" width="10.3076923076923" style="18" customWidth="1"/>
+    <col min="11" max="11" width="10.3076923076923" style="17" customWidth="1"/>
+    <col min="12" max="12" width="15.1538461538462" style="17" customWidth="1"/>
+    <col min="13" max="13" width="22.4615384615385" style="17" customWidth="1"/>
+    <col min="14" max="14" width="12.7692307692308" style="17" customWidth="1"/>
+    <col min="15" max="16" width="15.1538461538462" style="17" customWidth="1"/>
+    <col min="17" max="17" width="18.6923076923077" style="17" customWidth="1"/>
+    <col min="18" max="18" width="12.7692307692308" style="17" customWidth="1"/>
+    <col min="19" max="20" width="15.1538461538462" style="17" customWidth="1"/>
+    <col min="21" max="21" width="24.8461538461538" style="17" customWidth="1"/>
+    <col min="22" max="22" width="12.7692307692308" style="17" customWidth="1"/>
     <col min="23" max="23" width="10.3076923076923" customWidth="1"/>
     <col min="24" max="24" width="15.1538461538462" customWidth="1"/>
     <col min="25" max="25" width="41.8461538461538" customWidth="1"/>
@@ -1706,16 +1724,16 @@
       <c r="R1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="T1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="U1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="V1" s="11" t="s">
         <v>5</v>
       </c>
       <c r="W1" s="7" t="s">
@@ -1786,16 +1804,16 @@
       <c r="R2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="10" t="s">
+      <c r="T2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="U2" s="10" t="s">
+      <c r="U2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="V2" s="10" t="s">
+      <c r="V2" s="11" t="s">
         <v>12</v>
       </c>
       <c r="W2" s="7" t="s">
@@ -1858,14 +1876,14 @@
       <c r="R3" s="9">
         <v>0</v>
       </c>
-      <c r="S3" s="10">
-        <v>1</v>
-      </c>
-      <c r="T3" s="10">
-        <v>0</v>
-      </c>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10">
+      <c r="S3" s="11">
+        <v>1</v>
+      </c>
+      <c r="T3" s="11">
+        <v>0</v>
+      </c>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11">
         <v>0</v>
       </c>
       <c r="W3" s="7">
@@ -1926,14 +1944,14 @@
       <c r="R4" s="9">
         <v>0</v>
       </c>
-      <c r="S4" s="10">
-        <v>0</v>
-      </c>
-      <c r="T4" s="10">
-        <v>1</v>
-      </c>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10">
+      <c r="S4" s="11">
+        <v>0</v>
+      </c>
+      <c r="T4" s="11">
+        <v>1</v>
+      </c>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11">
         <v>0</v>
       </c>
       <c r="W4" s="7">
@@ -1994,14 +2012,14 @@
       <c r="R5" s="9">
         <v>0</v>
       </c>
-      <c r="S5" s="10">
-        <v>0</v>
-      </c>
-      <c r="T5" s="10">
-        <v>1</v>
-      </c>
-      <c r="U5" s="10"/>
-      <c r="V5" s="10">
+      <c r="S5" s="11">
+        <v>0</v>
+      </c>
+      <c r="T5" s="11">
+        <v>1</v>
+      </c>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11">
         <v>0</v>
       </c>
       <c r="W5" s="7">
@@ -2062,14 +2080,14 @@
       <c r="R6" s="9">
         <v>1</v>
       </c>
-      <c r="S6" s="10">
-        <v>1</v>
-      </c>
-      <c r="T6" s="10">
-        <v>1</v>
-      </c>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10">
+      <c r="S6" s="11">
+        <v>1</v>
+      </c>
+      <c r="T6" s="11">
+        <v>1</v>
+      </c>
+      <c r="U6" s="11"/>
+      <c r="V6" s="11">
         <v>1</v>
       </c>
       <c r="W6" s="7">
@@ -2130,14 +2148,14 @@
       <c r="R7" s="9">
         <v>0</v>
       </c>
-      <c r="S7" s="10">
-        <v>0</v>
-      </c>
-      <c r="T7" s="10">
-        <v>1</v>
-      </c>
-      <c r="U7" s="10"/>
-      <c r="V7" s="10">
+      <c r="S7" s="11">
+        <v>0</v>
+      </c>
+      <c r="T7" s="11">
+        <v>1</v>
+      </c>
+      <c r="U7" s="11"/>
+      <c r="V7" s="11">
         <v>0</v>
       </c>
       <c r="W7" s="7">
@@ -2198,14 +2216,14 @@
       <c r="R8" s="9">
         <v>1</v>
       </c>
-      <c r="S8" s="10">
-        <v>0</v>
-      </c>
-      <c r="T8" s="10">
-        <v>1</v>
-      </c>
-      <c r="U8" s="10"/>
-      <c r="V8" s="10">
+      <c r="S8" s="11">
+        <v>0</v>
+      </c>
+      <c r="T8" s="11">
+        <v>1</v>
+      </c>
+      <c r="U8" s="11"/>
+      <c r="V8" s="11">
         <v>1</v>
       </c>
       <c r="W8" s="7" t="s">
@@ -2266,14 +2284,14 @@
       <c r="R9" s="9">
         <v>1</v>
       </c>
-      <c r="S9" s="10">
-        <v>0</v>
-      </c>
-      <c r="T9" s="10">
-        <v>1</v>
-      </c>
-      <c r="U9" s="10"/>
-      <c r="V9" s="10">
+      <c r="S9" s="11">
+        <v>0</v>
+      </c>
+      <c r="T9" s="11">
+        <v>1</v>
+      </c>
+      <c r="U9" s="11"/>
+      <c r="V9" s="11">
         <v>1</v>
       </c>
       <c r="W9" s="7" t="s">
@@ -2334,14 +2352,14 @@
       <c r="R10" s="9">
         <v>0</v>
       </c>
-      <c r="S10" s="10">
-        <v>0</v>
-      </c>
-      <c r="T10" s="10">
-        <v>1</v>
-      </c>
-      <c r="U10" s="10"/>
-      <c r="V10" s="10">
+      <c r="S10" s="11">
+        <v>0</v>
+      </c>
+      <c r="T10" s="11">
+        <v>1</v>
+      </c>
+      <c r="U10" s="11"/>
+      <c r="V10" s="11">
         <v>0</v>
       </c>
       <c r="W10" s="7">
@@ -2402,14 +2420,14 @@
       <c r="R11" s="9">
         <v>1</v>
       </c>
-      <c r="S11" s="10">
-        <v>0</v>
-      </c>
-      <c r="T11" s="10">
-        <v>1</v>
-      </c>
-      <c r="U11" s="10"/>
-      <c r="V11" s="10">
+      <c r="S11" s="11">
+        <v>0</v>
+      </c>
+      <c r="T11" s="11">
+        <v>1</v>
+      </c>
+      <c r="U11" s="11"/>
+      <c r="V11" s="11">
         <v>1</v>
       </c>
       <c r="W11" s="7">
@@ -2470,14 +2488,14 @@
       <c r="R12" s="9">
         <v>0</v>
       </c>
-      <c r="S12" s="10">
-        <v>0</v>
-      </c>
-      <c r="T12" s="10">
-        <v>1</v>
-      </c>
-      <c r="U12" s="10"/>
-      <c r="V12" s="10">
+      <c r="S12" s="11">
+        <v>0</v>
+      </c>
+      <c r="T12" s="11">
+        <v>1</v>
+      </c>
+      <c r="U12" s="11"/>
+      <c r="V12" s="11">
         <v>0</v>
       </c>
       <c r="W12" s="7">
@@ -2538,14 +2556,14 @@
       <c r="R13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U13" s="10"/>
-      <c r="V13" s="10" t="s">
+      <c r="S13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U13" s="11"/>
+      <c r="V13" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W13" s="7" t="s">
@@ -2606,14 +2624,14 @@
       <c r="R14" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S14" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T14" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U14" s="10"/>
-      <c r="V14" s="10" t="s">
+      <c r="S14" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T14" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U14" s="11"/>
+      <c r="V14" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W14" s="7" t="s">
@@ -2674,14 +2692,14 @@
       <c r="R15" s="9">
         <v>1</v>
       </c>
-      <c r="S15" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T15" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U15" s="10"/>
-      <c r="V15" s="10" t="s">
+      <c r="S15" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T15" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W15" s="7" t="s">
@@ -2742,14 +2760,14 @@
       <c r="R16" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S16" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T16" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U16" s="10"/>
-      <c r="V16" s="10" t="s">
+      <c r="S16" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T16" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W16" s="7">
@@ -2810,16 +2828,16 @@
       <c r="R17" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S17" s="10">
-        <v>1</v>
-      </c>
-      <c r="T17" s="10">
-        <v>1</v>
-      </c>
-      <c r="U17" s="10" t="s">
+      <c r="S17" s="11">
+        <v>1</v>
+      </c>
+      <c r="T17" s="11">
+        <v>1</v>
+      </c>
+      <c r="U17" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="V17" s="10">
+      <c r="V17" s="11">
         <v>0</v>
       </c>
       <c r="W17" s="7" t="s">
@@ -2880,14 +2898,14 @@
       <c r="R18" s="9">
         <v>0</v>
       </c>
-      <c r="S18" s="10">
-        <v>0</v>
-      </c>
-      <c r="T18" s="10">
-        <v>1</v>
-      </c>
-      <c r="U18" s="10"/>
-      <c r="V18" s="10">
+      <c r="S18" s="11">
+        <v>0</v>
+      </c>
+      <c r="T18" s="11">
+        <v>1</v>
+      </c>
+      <c r="U18" s="11"/>
+      <c r="V18" s="11">
         <v>0</v>
       </c>
       <c r="W18" s="7">
@@ -2948,14 +2966,14 @@
       <c r="R19" s="9">
         <v>0</v>
       </c>
-      <c r="S19" s="10">
-        <v>1</v>
-      </c>
-      <c r="T19" s="10">
-        <v>1</v>
-      </c>
-      <c r="U19" s="10"/>
-      <c r="V19" s="10">
+      <c r="S19" s="11">
+        <v>1</v>
+      </c>
+      <c r="T19" s="11">
+        <v>1</v>
+      </c>
+      <c r="U19" s="11"/>
+      <c r="V19" s="11">
         <v>0</v>
       </c>
       <c r="W19" s="7">
@@ -3016,14 +3034,14 @@
       <c r="R20" s="9">
         <v>0</v>
       </c>
-      <c r="S20" s="10">
-        <v>0</v>
-      </c>
-      <c r="T20" s="10">
-        <v>1</v>
-      </c>
-      <c r="U20" s="10"/>
-      <c r="V20" s="10">
+      <c r="S20" s="11">
+        <v>0</v>
+      </c>
+      <c r="T20" s="11">
+        <v>1</v>
+      </c>
+      <c r="U20" s="11"/>
+      <c r="V20" s="11">
         <v>0</v>
       </c>
       <c r="W20" s="7">
@@ -3041,7 +3059,7 @@
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="19" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="2">
@@ -3084,14 +3102,14 @@
       <c r="R21" s="9">
         <v>1</v>
       </c>
-      <c r="S21" s="10">
-        <v>0</v>
-      </c>
-      <c r="T21" s="10">
-        <v>1</v>
-      </c>
-      <c r="U21" s="10"/>
-      <c r="V21" s="10">
+      <c r="S21" s="11">
+        <v>0</v>
+      </c>
+      <c r="T21" s="11">
+        <v>1</v>
+      </c>
+      <c r="U21" s="11"/>
+      <c r="V21" s="11">
         <v>1</v>
       </c>
       <c r="W21" s="7" t="s">
@@ -3109,7 +3127,7 @@
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="19" t="s">
         <v>35</v>
       </c>
       <c r="C22" s="2">
@@ -3152,14 +3170,14 @@
       <c r="R22" s="9">
         <v>1</v>
       </c>
-      <c r="S22" s="10">
-        <v>1</v>
-      </c>
-      <c r="T22" s="10">
-        <v>1</v>
-      </c>
-      <c r="U22" s="10"/>
-      <c r="V22" s="10">
+      <c r="S22" s="11">
+        <v>1</v>
+      </c>
+      <c r="T22" s="11">
+        <v>1</v>
+      </c>
+      <c r="U22" s="11"/>
+      <c r="V22" s="11">
         <v>1</v>
       </c>
       <c r="W22" s="7" t="s">
@@ -3177,7 +3195,7 @@
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="19" t="s">
         <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -3220,14 +3238,14 @@
       <c r="R23" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S23" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T23" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U23" s="10"/>
-      <c r="V23" s="10" t="s">
+      <c r="S23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U23" s="11"/>
+      <c r="V23" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W23" s="7">
@@ -3243,7 +3261,7 @@
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="19" t="s">
         <v>37</v>
       </c>
       <c r="C24" s="2">
@@ -3286,14 +3304,14 @@
       <c r="R24" s="9">
         <v>1</v>
       </c>
-      <c r="S24" s="10">
-        <v>0</v>
-      </c>
-      <c r="T24" s="10">
-        <v>0</v>
-      </c>
-      <c r="U24" s="10"/>
-      <c r="V24" s="10">
+      <c r="S24" s="11">
+        <v>0</v>
+      </c>
+      <c r="T24" s="11">
+        <v>0</v>
+      </c>
+      <c r="U24" s="11"/>
+      <c r="V24" s="11">
         <v>1</v>
       </c>
       <c r="W24" s="7">
@@ -3354,14 +3372,14 @@
       <c r="R25" s="9">
         <v>0</v>
       </c>
-      <c r="S25" s="10">
-        <v>0</v>
-      </c>
-      <c r="T25" s="10">
-        <v>1</v>
-      </c>
-      <c r="U25" s="10"/>
-      <c r="V25" s="10">
+      <c r="S25" s="11">
+        <v>0</v>
+      </c>
+      <c r="T25" s="11">
+        <v>1</v>
+      </c>
+      <c r="U25" s="11"/>
+      <c r="V25" s="11">
         <v>0</v>
       </c>
       <c r="W25" s="7">
@@ -3422,14 +3440,14 @@
       <c r="R26" s="9">
         <v>0</v>
       </c>
-      <c r="S26" s="10">
-        <v>1</v>
-      </c>
-      <c r="T26" s="10">
-        <v>1</v>
-      </c>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10">
+      <c r="S26" s="11">
+        <v>1</v>
+      </c>
+      <c r="T26" s="11">
+        <v>1</v>
+      </c>
+      <c r="U26" s="11"/>
+      <c r="V26" s="11">
         <v>0</v>
       </c>
       <c r="W26" s="7">
@@ -3490,14 +3508,14 @@
       <c r="R27" s="9">
         <v>1</v>
       </c>
-      <c r="S27" s="10">
-        <v>1</v>
-      </c>
-      <c r="T27" s="10">
-        <v>1</v>
-      </c>
-      <c r="U27" s="10"/>
-      <c r="V27" s="10">
+      <c r="S27" s="11">
+        <v>1</v>
+      </c>
+      <c r="T27" s="11">
+        <v>1</v>
+      </c>
+      <c r="U27" s="11"/>
+      <c r="V27" s="11">
         <v>1</v>
       </c>
       <c r="W27" s="7">
@@ -3558,14 +3576,14 @@
       <c r="R28" s="9">
         <v>1</v>
       </c>
-      <c r="S28" s="10">
-        <v>0</v>
-      </c>
-      <c r="T28" s="10">
-        <v>1</v>
-      </c>
-      <c r="U28" s="10"/>
-      <c r="V28" s="10">
+      <c r="S28" s="11">
+        <v>0</v>
+      </c>
+      <c r="T28" s="11">
+        <v>1</v>
+      </c>
+      <c r="U28" s="11"/>
+      <c r="V28" s="11">
         <v>1</v>
       </c>
       <c r="W28" s="7">
@@ -3626,14 +3644,14 @@
       <c r="R29" s="9">
         <v>0</v>
       </c>
-      <c r="S29" s="10">
-        <v>0</v>
-      </c>
-      <c r="T29" s="10">
-        <v>1</v>
-      </c>
-      <c r="U29" s="10"/>
-      <c r="V29" s="10">
+      <c r="S29" s="11">
+        <v>0</v>
+      </c>
+      <c r="T29" s="11">
+        <v>1</v>
+      </c>
+      <c r="U29" s="11"/>
+      <c r="V29" s="11">
         <v>0</v>
       </c>
       <c r="W29" s="7">
@@ -3694,14 +3712,14 @@
       <c r="R30" s="9">
         <v>0</v>
       </c>
-      <c r="S30" s="10">
-        <v>0</v>
-      </c>
-      <c r="T30" s="10">
-        <v>1</v>
-      </c>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10">
+      <c r="S30" s="11">
+        <v>0</v>
+      </c>
+      <c r="T30" s="11">
+        <v>1</v>
+      </c>
+      <c r="U30" s="11"/>
+      <c r="V30" s="11">
         <v>0</v>
       </c>
       <c r="W30" s="7">
@@ -3762,14 +3780,14 @@
       <c r="R31" s="9">
         <v>0</v>
       </c>
-      <c r="S31" s="10">
-        <v>0</v>
-      </c>
-      <c r="T31" s="10">
-        <v>1</v>
-      </c>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10">
+      <c r="S31" s="11">
+        <v>0</v>
+      </c>
+      <c r="T31" s="11">
+        <v>1</v>
+      </c>
+      <c r="U31" s="11"/>
+      <c r="V31" s="11">
         <v>0</v>
       </c>
       <c r="W31" s="7">
@@ -3830,14 +3848,14 @@
       <c r="R32" s="9">
         <v>0</v>
       </c>
-      <c r="S32" s="10">
-        <v>0</v>
-      </c>
-      <c r="T32" s="10">
-        <v>1</v>
-      </c>
-      <c r="U32" s="10"/>
-      <c r="V32" s="10">
+      <c r="S32" s="11">
+        <v>0</v>
+      </c>
+      <c r="T32" s="11">
+        <v>1</v>
+      </c>
+      <c r="U32" s="11"/>
+      <c r="V32" s="11">
         <v>0</v>
       </c>
       <c r="W32" s="7">
@@ -3932,16 +3950,16 @@
       <c r="R1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="T1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="U1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="V1" s="11" t="s">
         <v>5</v>
       </c>
       <c r="W1" s="7" t="s">
@@ -4012,16 +4030,16 @@
       <c r="R2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="10" t="s">
+      <c r="T2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="U2" s="10" t="s">
+      <c r="U2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="V2" s="10" t="s">
+      <c r="V2" s="11" t="s">
         <v>12</v>
       </c>
       <c r="W2" s="7" t="s">
@@ -4084,14 +4102,14 @@
       <c r="R3" s="9">
         <v>1</v>
       </c>
-      <c r="S3" s="10">
-        <v>1</v>
-      </c>
-      <c r="T3" s="10">
-        <v>1</v>
-      </c>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10">
+      <c r="S3" s="11">
+        <v>1</v>
+      </c>
+      <c r="T3" s="11">
+        <v>1</v>
+      </c>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11">
         <v>1</v>
       </c>
       <c r="W3" s="7">
@@ -4152,14 +4170,14 @@
       <c r="R4" s="9">
         <v>0</v>
       </c>
-      <c r="S4" s="10">
-        <v>0</v>
-      </c>
-      <c r="T4" s="10">
-        <v>1</v>
-      </c>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10">
+      <c r="S4" s="11">
+        <v>0</v>
+      </c>
+      <c r="T4" s="11">
+        <v>1</v>
+      </c>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11">
         <v>0</v>
       </c>
       <c r="W4" s="7">
@@ -4220,14 +4238,14 @@
       <c r="R5" s="9">
         <v>1</v>
       </c>
-      <c r="S5" s="10">
-        <v>1</v>
-      </c>
-      <c r="T5" s="10">
-        <v>1</v>
-      </c>
-      <c r="U5" s="10"/>
-      <c r="V5" s="10">
+      <c r="S5" s="11">
+        <v>1</v>
+      </c>
+      <c r="T5" s="11">
+        <v>1</v>
+      </c>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11">
         <v>1</v>
       </c>
       <c r="W5" s="7" t="s">
@@ -4288,14 +4306,14 @@
       <c r="R6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S6" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T6" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10" t="s">
+      <c r="S6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U6" s="11"/>
+      <c r="V6" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W6" s="7">
@@ -4358,14 +4376,14 @@
       <c r="R7" s="9">
         <v>0</v>
       </c>
-      <c r="S7" s="10">
-        <v>1</v>
-      </c>
-      <c r="T7" s="10">
-        <v>1</v>
-      </c>
-      <c r="U7" s="10"/>
-      <c r="V7" s="10">
+      <c r="S7" s="11">
+        <v>1</v>
+      </c>
+      <c r="T7" s="11">
+        <v>1</v>
+      </c>
+      <c r="U7" s="11"/>
+      <c r="V7" s="11">
         <v>0</v>
       </c>
       <c r="W7" s="7" t="s">
@@ -4428,16 +4446,16 @@
       <c r="R8" s="9">
         <v>1</v>
       </c>
-      <c r="S8" s="10">
-        <v>1</v>
-      </c>
-      <c r="T8" s="10">
-        <v>1</v>
-      </c>
-      <c r="U8" s="10" t="s">
+      <c r="S8" s="11">
+        <v>1</v>
+      </c>
+      <c r="T8" s="11">
+        <v>1</v>
+      </c>
+      <c r="U8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="V8" s="10">
+      <c r="V8" s="11">
         <v>1</v>
       </c>
       <c r="W8" s="7" t="s">
@@ -4502,16 +4520,16 @@
       <c r="R9" s="9">
         <v>1</v>
       </c>
-      <c r="S9" s="10">
-        <v>1</v>
-      </c>
-      <c r="T9" s="10">
-        <v>1</v>
-      </c>
-      <c r="U9" s="10" t="s">
+      <c r="S9" s="11">
+        <v>1</v>
+      </c>
+      <c r="T9" s="11">
+        <v>1</v>
+      </c>
+      <c r="U9" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="V9" s="10">
+      <c r="V9" s="11">
         <v>1</v>
       </c>
       <c r="W9" s="7" t="s">
@@ -4576,16 +4594,16 @@
       <c r="R10" s="9">
         <v>1</v>
       </c>
-      <c r="S10" s="10">
-        <v>1</v>
-      </c>
-      <c r="T10" s="10">
-        <v>1</v>
-      </c>
-      <c r="U10" s="10" t="s">
+      <c r="S10" s="11">
+        <v>1</v>
+      </c>
+      <c r="T10" s="11">
+        <v>1</v>
+      </c>
+      <c r="U10" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="V10" s="10">
+      <c r="V10" s="11">
         <v>0</v>
       </c>
       <c r="W10" s="7">
@@ -4652,14 +4670,14 @@
       <c r="R11" s="9">
         <v>0</v>
       </c>
-      <c r="S11" s="10">
-        <v>1</v>
-      </c>
-      <c r="T11" s="10">
-        <v>1</v>
-      </c>
-      <c r="U11" s="10"/>
-      <c r="V11" s="10">
+      <c r="S11" s="11">
+        <v>1</v>
+      </c>
+      <c r="T11" s="11">
+        <v>1</v>
+      </c>
+      <c r="U11" s="11"/>
+      <c r="V11" s="11">
         <v>0</v>
       </c>
       <c r="W11" s="7">
@@ -4720,14 +4738,14 @@
       <c r="R12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S12" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T12" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U12" s="10"/>
-      <c r="V12" s="10" t="s">
+      <c r="S12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U12" s="11"/>
+      <c r="V12" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W12" s="7">
@@ -4790,14 +4808,14 @@
       <c r="R13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U13" s="10"/>
-      <c r="V13" s="10" t="s">
+      <c r="S13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U13" s="11"/>
+      <c r="V13" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W13" s="7">
@@ -4864,14 +4882,14 @@
       <c r="R14" s="9">
         <v>0</v>
       </c>
-      <c r="S14" s="10">
-        <v>1</v>
-      </c>
-      <c r="T14" s="10">
-        <v>1</v>
-      </c>
-      <c r="U14" s="10"/>
-      <c r="V14" s="10">
+      <c r="S14" s="11">
+        <v>1</v>
+      </c>
+      <c r="T14" s="11">
+        <v>1</v>
+      </c>
+      <c r="U14" s="11"/>
+      <c r="V14" s="11">
         <v>0</v>
       </c>
       <c r="W14" s="7">
@@ -4934,14 +4952,14 @@
       <c r="R15" s="9">
         <v>1</v>
       </c>
-      <c r="S15" s="10">
-        <v>1</v>
-      </c>
-      <c r="T15" s="10">
-        <v>1</v>
-      </c>
-      <c r="U15" s="10"/>
-      <c r="V15" s="10">
+      <c r="S15" s="11">
+        <v>1</v>
+      </c>
+      <c r="T15" s="11">
+        <v>1</v>
+      </c>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11">
         <v>1</v>
       </c>
       <c r="W15" s="7" t="s">
@@ -5002,14 +5020,14 @@
       <c r="R16" s="9">
         <v>0</v>
       </c>
-      <c r="S16" s="10">
-        <v>1</v>
-      </c>
-      <c r="T16" s="10">
-        <v>1</v>
-      </c>
-      <c r="U16" s="10"/>
-      <c r="V16" s="10">
+      <c r="S16" s="11">
+        <v>1</v>
+      </c>
+      <c r="T16" s="11">
+        <v>1</v>
+      </c>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11">
         <v>0</v>
       </c>
       <c r="W16" s="7" t="s">
@@ -5072,14 +5090,14 @@
       <c r="R17" s="9">
         <v>1</v>
       </c>
-      <c r="S17" s="10">
-        <v>1</v>
-      </c>
-      <c r="T17" s="10">
-        <v>1</v>
-      </c>
-      <c r="U17" s="10"/>
-      <c r="V17" s="10">
+      <c r="S17" s="11">
+        <v>1</v>
+      </c>
+      <c r="T17" s="11">
+        <v>1</v>
+      </c>
+      <c r="U17" s="11"/>
+      <c r="V17" s="11">
         <v>1</v>
       </c>
       <c r="W17" s="7">
@@ -5140,14 +5158,14 @@
       <c r="R18" s="9">
         <v>1</v>
       </c>
-      <c r="S18" s="10">
-        <v>1</v>
-      </c>
-      <c r="T18" s="10">
-        <v>1</v>
-      </c>
-      <c r="U18" s="10"/>
-      <c r="V18" s="10">
+      <c r="S18" s="11">
+        <v>1</v>
+      </c>
+      <c r="T18" s="11">
+        <v>1</v>
+      </c>
+      <c r="U18" s="11"/>
+      <c r="V18" s="11">
         <v>1</v>
       </c>
       <c r="W18" s="7">
@@ -5208,14 +5226,14 @@
       <c r="R19" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S19" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T19" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U19" s="10"/>
-      <c r="V19" s="10" t="s">
+      <c r="S19" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T19" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U19" s="11"/>
+      <c r="V19" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W19" s="7">
@@ -5276,14 +5294,14 @@
       <c r="R20" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S20" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T20" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U20" s="10"/>
-      <c r="V20" s="10" t="s">
+      <c r="S20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U20" s="11"/>
+      <c r="V20" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W20" s="7">
@@ -5301,7 +5319,7 @@
       <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="16" t="s">
         <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -5344,14 +5362,14 @@
       <c r="R21" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S21" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T21" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U21" s="10"/>
-      <c r="V21" s="10" t="s">
+      <c r="S21" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T21" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U21" s="11"/>
+      <c r="V21" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W21" s="7">
@@ -5412,14 +5430,14 @@
       <c r="R22" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S22" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T22" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U22" s="10"/>
-      <c r="V22" s="10" t="s">
+      <c r="S22" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T22" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U22" s="11"/>
+      <c r="V22" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W22" s="7">
@@ -5480,14 +5498,14 @@
       <c r="R23" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S23" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T23" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U23" s="10"/>
-      <c r="V23" s="10" t="s">
+      <c r="S23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U23" s="11"/>
+      <c r="V23" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W23" s="7">
@@ -5548,14 +5566,14 @@
       <c r="R24" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S24" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T24" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U24" s="10"/>
-      <c r="V24" s="10" t="s">
+      <c r="S24" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T24" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U24" s="11"/>
+      <c r="V24" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W24" s="7">
@@ -5618,14 +5636,14 @@
       <c r="R25" s="9">
         <v>1</v>
       </c>
-      <c r="S25" s="10">
-        <v>1</v>
-      </c>
-      <c r="T25" s="10">
-        <v>1</v>
-      </c>
-      <c r="U25" s="10"/>
-      <c r="V25" s="10">
+      <c r="S25" s="11">
+        <v>1</v>
+      </c>
+      <c r="T25" s="11">
+        <v>1</v>
+      </c>
+      <c r="U25" s="11"/>
+      <c r="V25" s="11">
         <v>1</v>
       </c>
       <c r="W25" s="7" t="s">
@@ -5686,14 +5704,14 @@
       <c r="R26" s="9">
         <v>1</v>
       </c>
-      <c r="S26" s="10">
-        <v>1</v>
-      </c>
-      <c r="T26" s="10">
-        <v>0</v>
-      </c>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10">
+      <c r="S26" s="11">
+        <v>1</v>
+      </c>
+      <c r="T26" s="11">
+        <v>0</v>
+      </c>
+      <c r="U26" s="11"/>
+      <c r="V26" s="11">
         <v>1</v>
       </c>
       <c r="W26" s="7">
@@ -5756,14 +5774,14 @@
       <c r="R27" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S27" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T27" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U27" s="10"/>
-      <c r="V27" s="10" t="s">
+      <c r="S27" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T27" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U27" s="11"/>
+      <c r="V27" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W27" s="7" t="s">
@@ -5824,14 +5842,14 @@
       <c r="R28" s="9">
         <v>1</v>
       </c>
-      <c r="S28" s="10">
-        <v>1</v>
-      </c>
-      <c r="T28" s="10">
-        <v>1</v>
-      </c>
-      <c r="U28" s="10"/>
-      <c r="V28" s="10">
+      <c r="S28" s="11">
+        <v>1</v>
+      </c>
+      <c r="T28" s="11">
+        <v>1</v>
+      </c>
+      <c r="U28" s="11"/>
+      <c r="V28" s="11">
         <v>1</v>
       </c>
       <c r="W28" s="7">
@@ -5892,14 +5910,14 @@
       <c r="R29" s="9">
         <v>1</v>
       </c>
-      <c r="S29" s="10">
-        <v>1</v>
-      </c>
-      <c r="T29" s="10">
-        <v>0</v>
-      </c>
-      <c r="U29" s="10"/>
-      <c r="V29" s="10">
+      <c r="S29" s="11">
+        <v>1</v>
+      </c>
+      <c r="T29" s="11">
+        <v>0</v>
+      </c>
+      <c r="U29" s="11"/>
+      <c r="V29" s="11">
         <v>1</v>
       </c>
       <c r="W29" s="7" t="s">
@@ -5958,14 +5976,14 @@
       <c r="R30" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="S30" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="T30" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10" t="s">
+      <c r="S30" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="T30" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="U30" s="11"/>
+      <c r="V30" s="11" t="s">
         <v>20</v>
       </c>
       <c r="W30" s="7">
@@ -6026,14 +6044,14 @@
       <c r="R31" s="9">
         <v>1</v>
       </c>
-      <c r="S31" s="10">
-        <v>1</v>
-      </c>
-      <c r="T31" s="10">
-        <v>1</v>
-      </c>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10">
+      <c r="S31" s="11">
+        <v>1</v>
+      </c>
+      <c r="T31" s="11">
+        <v>1</v>
+      </c>
+      <c r="U31" s="11"/>
+      <c r="V31" s="11">
         <v>1</v>
       </c>
       <c r="W31" s="7">
@@ -6094,14 +6112,14 @@
       <c r="R32" s="9">
         <v>1</v>
       </c>
-      <c r="S32" s="10">
-        <v>1</v>
-      </c>
-      <c r="T32" s="10">
-        <v>1</v>
-      </c>
-      <c r="U32" s="10"/>
-      <c r="V32" s="10">
+      <c r="S32" s="11">
+        <v>1</v>
+      </c>
+      <c r="T32" s="11">
+        <v>1</v>
+      </c>
+      <c r="U32" s="11"/>
+      <c r="V32" s="11">
         <v>1</v>
       </c>
       <c r="W32" s="7">
@@ -6162,14 +6180,14 @@
       <c r="R33" s="9">
         <v>1</v>
       </c>
-      <c r="S33" s="10">
-        <v>1</v>
-      </c>
-      <c r="T33" s="10">
-        <v>1</v>
-      </c>
-      <c r="U33" s="10"/>
-      <c r="V33" s="10">
+      <c r="S33" s="11">
+        <v>1</v>
+      </c>
+      <c r="T33" s="11">
+        <v>1</v>
+      </c>
+      <c r="U33" s="11"/>
+      <c r="V33" s="11">
         <v>1</v>
       </c>
       <c r="W33" s="7">
@@ -6230,14 +6248,14 @@
       <c r="R34" s="9">
         <v>1</v>
       </c>
-      <c r="S34" s="10">
-        <v>0</v>
-      </c>
-      <c r="T34" s="10">
-        <v>0</v>
-      </c>
-      <c r="U34" s="10"/>
-      <c r="V34" s="10">
+      <c r="S34" s="11">
+        <v>0</v>
+      </c>
+      <c r="T34" s="11">
+        <v>0</v>
+      </c>
+      <c r="U34" s="11"/>
+      <c r="V34" s="11">
         <v>1</v>
       </c>
       <c r="W34" s="7">
@@ -6298,14 +6316,14 @@
       <c r="R35" s="9">
         <v>0</v>
       </c>
-      <c r="S35" s="10">
-        <v>0</v>
-      </c>
-      <c r="T35" s="10">
-        <v>1</v>
-      </c>
-      <c r="U35" s="10"/>
-      <c r="V35" s="10">
+      <c r="S35" s="11">
+        <v>0</v>
+      </c>
+      <c r="T35" s="11">
+        <v>1</v>
+      </c>
+      <c r="U35" s="11"/>
+      <c r="V35" s="11">
         <v>0</v>
       </c>
       <c r="W35" s="7">
@@ -6323,7 +6341,7 @@
       <c r="A36" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="16" t="s">
         <v>100</v>
       </c>
       <c r="C36" s="2">
@@ -6366,14 +6384,14 @@
       <c r="R36" s="9">
         <v>1</v>
       </c>
-      <c r="S36" s="10">
-        <v>1</v>
-      </c>
-      <c r="T36" s="10">
-        <v>1</v>
-      </c>
-      <c r="U36" s="10"/>
-      <c r="V36" s="10">
+      <c r="S36" s="11">
+        <v>1</v>
+      </c>
+      <c r="T36" s="11">
+        <v>1</v>
+      </c>
+      <c r="U36" s="11"/>
+      <c r="V36" s="11">
         <v>1</v>
       </c>
       <c r="W36" s="7">
@@ -6396,19 +6414,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AH7"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <cols>
     <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
-    <col min="11" max="18" width="20" customWidth="1"/>
-    <col min="19" max="19" width="10.3076923076923" customWidth="1"/>
-    <col min="20" max="20" width="15.1538461538462" customWidth="1"/>
-    <col min="21" max="21" width="10.3076923076923" customWidth="1"/>
-    <col min="22" max="22" width="12.7692307692308" customWidth="1"/>
+    <col min="11" max="26" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30">
+    <row r="1" spans="1:34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6462,43 +6476,55 @@
         <v>101</v>
       </c>
       <c r="S1" s="9" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="T1" s="9" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="V1" s="9" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="W1" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="X1" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y1" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z1" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="X1" s="10" t="s">
+      <c r="AB1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="Y1" s="10" t="s">
+      <c r="AC1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="Z1" s="10" t="s">
+      <c r="AD1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="AA1" s="7" t="s">
+      <c r="AE1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AB1" s="7" t="s">
+      <c r="AF1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AC1" s="7" t="s">
+      <c r="AG1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AD1" s="7" t="s">
+      <c r="AH1" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:30">
+    <row r="2" spans="1:34">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -6529,7 +6555,7 @@
       <c r="J2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="12" t="s">
         <v>9</v>
       </c>
       <c r="L2" s="7" t="s">
@@ -6577,25 +6603,37 @@
       <c r="Z2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="AA2" s="7" t="s">
+      <c r="AA2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="AB2" s="7" t="s">
+      <c r="AB2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="AC2" s="7" t="s">
+      <c r="AC2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="AD2" s="7" t="s">
+      <c r="AD2" s="11" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:30">
+      <c r="AE2" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="AG2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH2" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34">
       <c r="A3" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>20</v>
@@ -6617,14 +6655,14 @@
       <c r="J3" s="5">
         <v>0</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="K3" s="12" t="s">
         <v>20</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M3" s="7"/>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="O3" s="8">
@@ -6634,7 +6672,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="8"/>
-      <c r="R3" s="13">
+      <c r="R3" s="14">
         <v>0</v>
       </c>
       <c r="S3" s="9" t="s">
@@ -6653,29 +6691,39 @@
       <c r="X3" s="10">
         <v>1</v>
       </c>
-      <c r="Y3" s="10" t="s">
+      <c r="Y3" s="10"/>
+      <c r="Z3" s="15">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="AD3" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34">
+      <c r="A4" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="Z3" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AC3" s="7"/>
-      <c r="AD3" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30">
-      <c r="A4" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="B4" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -6697,14 +6745,14 @@
       <c r="J4" s="5">
         <v>0</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="K4" s="12" t="s">
         <v>20</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M4" s="7"/>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="13" t="s">
         <v>20</v>
       </c>
       <c r="O4" s="8">
@@ -6714,7 +6762,7 @@
         <v>1</v>
       </c>
       <c r="Q4" s="8"/>
-      <c r="R4" s="13">
+      <c r="R4" s="14">
         <v>0</v>
       </c>
       <c r="S4" s="9" t="s">
@@ -6728,32 +6776,42 @@
         <v>20</v>
       </c>
       <c r="W4" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4" s="10">
         <v>1</v>
       </c>
       <c r="Y4" s="10"/>
-      <c r="Z4" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AC4" s="7"/>
-      <c r="AD4" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:30">
+      <c r="Z4" s="15">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC4" s="11"/>
+      <c r="AD4" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34">
       <c r="A5" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>20</v>
@@ -6775,14 +6833,14 @@
       <c r="J5" s="5">
         <v>0</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="K5" s="12" t="s">
         <v>20</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M5" s="7"/>
-      <c r="N5" s="12" t="s">
+      <c r="N5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="O5" s="8">
@@ -6792,7 +6850,7 @@
         <v>1</v>
       </c>
       <c r="Q5" s="8"/>
-      <c r="R5" s="13">
+      <c r="R5" s="14">
         <v>0</v>
       </c>
       <c r="S5" s="9" t="s">
@@ -6806,32 +6864,42 @@
         <v>20</v>
       </c>
       <c r="W5" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X5" s="10">
         <v>1</v>
       </c>
       <c r="Y5" s="10"/>
-      <c r="Z5" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AC5" s="7"/>
-      <c r="AD5" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30">
+      <c r="Z5" s="15">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC5" s="11"/>
+      <c r="AD5" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34">
       <c r="A6" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -6853,14 +6921,14 @@
       <c r="J6" s="5">
         <v>0</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="12" t="s">
         <v>20</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M6" s="7"/>
-      <c r="N6" s="12" t="s">
+      <c r="N6" s="13" t="s">
         <v>20</v>
       </c>
       <c r="O6" s="8">
@@ -6870,7 +6938,7 @@
         <v>1</v>
       </c>
       <c r="Q6" s="8"/>
-      <c r="R6" s="13">
+      <c r="R6" s="14">
         <v>0</v>
       </c>
       <c r="S6" s="9" t="s">
@@ -6884,29 +6952,39 @@
         <v>20</v>
       </c>
       <c r="W6" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6" s="10">
         <v>1</v>
       </c>
       <c r="Y6" s="10"/>
-      <c r="Z6" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AC6" s="7"/>
-      <c r="AD6" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30">
+      <c r="Z6" s="15">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC6" s="11"/>
+      <c r="AD6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34">
       <c r="A7" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>
@@ -6931,14 +7009,14 @@
       <c r="J7" s="5">
         <v>0</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="12" t="s">
         <v>20</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M7" s="7"/>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="13" t="s">
         <v>20</v>
       </c>
       <c r="O7" s="8">
@@ -6948,7 +7026,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="8"/>
-      <c r="R7" s="13">
+      <c r="R7" s="14">
         <v>0</v>
       </c>
       <c r="S7" s="9" t="s">
@@ -6962,23 +7040,33 @@
         <v>20</v>
       </c>
       <c r="W7" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X7" s="10">
         <v>1</v>
       </c>
       <c r="Y7" s="10"/>
-      <c r="Z7" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AC7" s="7"/>
-      <c r="AD7" s="7" t="s">
+      <c r="Z7" s="15">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC7" s="11"/>
+      <c r="AD7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="7" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-06-11 11:23:47
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="112">
   <si>
     <t>招标方式</t>
   </si>
@@ -342,6 +342,12 @@
   </si>
   <si>
     <t>谈判采购（邀请）</t>
+  </si>
+  <si>
+    <t>直接采购（公开）</t>
+  </si>
+  <si>
+    <t>直接采购（邀请）</t>
   </si>
   <si>
     <t>邀请供应商</t>
@@ -525,7 +531,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -571,6 +577,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -934,7 +946,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -958,16 +970,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -976,89 +988,89 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1093,6 +1105,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1649,22 +1664,22 @@
   <cols>
     <col min="1" max="1" width="16.3846153846154" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="22.4615384615385" style="17" customWidth="1"/>
-    <col min="4" max="5" width="15.1538461538462" style="17" customWidth="1"/>
-    <col min="6" max="6" width="12.7692307692308" style="17" customWidth="1"/>
-    <col min="7" max="7" width="22.4615384615385" style="18" customWidth="1"/>
-    <col min="8" max="9" width="15.1538461538462" style="18" customWidth="1"/>
-    <col min="10" max="10" width="10.3076923076923" style="18" customWidth="1"/>
-    <col min="11" max="11" width="10.3076923076923" style="17" customWidth="1"/>
-    <col min="12" max="12" width="15.1538461538462" style="17" customWidth="1"/>
-    <col min="13" max="13" width="22.4615384615385" style="17" customWidth="1"/>
-    <col min="14" max="14" width="12.7692307692308" style="17" customWidth="1"/>
-    <col min="15" max="16" width="15.1538461538462" style="17" customWidth="1"/>
-    <col min="17" max="17" width="18.6923076923077" style="17" customWidth="1"/>
-    <col min="18" max="18" width="12.7692307692308" style="17" customWidth="1"/>
-    <col min="19" max="20" width="15.1538461538462" style="17" customWidth="1"/>
-    <col min="21" max="21" width="24.8461538461538" style="17" customWidth="1"/>
-    <col min="22" max="22" width="12.7692307692308" style="17" customWidth="1"/>
+    <col min="3" max="3" width="22.4615384615385" style="18" customWidth="1"/>
+    <col min="4" max="5" width="15.1538461538462" style="18" customWidth="1"/>
+    <col min="6" max="6" width="12.7692307692308" style="18" customWidth="1"/>
+    <col min="7" max="7" width="22.4615384615385" style="19" customWidth="1"/>
+    <col min="8" max="9" width="15.1538461538462" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.3076923076923" style="19" customWidth="1"/>
+    <col min="11" max="11" width="10.3076923076923" style="18" customWidth="1"/>
+    <col min="12" max="12" width="15.1538461538462" style="18" customWidth="1"/>
+    <col min="13" max="13" width="22.4615384615385" style="18" customWidth="1"/>
+    <col min="14" max="14" width="12.7692307692308" style="18" customWidth="1"/>
+    <col min="15" max="16" width="15.1538461538462" style="18" customWidth="1"/>
+    <col min="17" max="17" width="18.6923076923077" style="18" customWidth="1"/>
+    <col min="18" max="18" width="12.7692307692308" style="18" customWidth="1"/>
+    <col min="19" max="20" width="15.1538461538462" style="18" customWidth="1"/>
+    <col min="21" max="21" width="24.8461538461538" style="18" customWidth="1"/>
+    <col min="22" max="22" width="12.7692307692308" style="18" customWidth="1"/>
     <col min="23" max="23" width="10.3076923076923" customWidth="1"/>
     <col min="24" max="24" width="15.1538461538462" customWidth="1"/>
     <col min="25" max="25" width="41.8461538461538" customWidth="1"/>
@@ -3059,7 +3074,7 @@
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="20" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="2">
@@ -3127,7 +3142,7 @@
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="20" t="s">
         <v>35</v>
       </c>
       <c r="C22" s="2">
@@ -3195,7 +3210,7 @@
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -3261,7 +3276,7 @@
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="20" t="s">
         <v>37</v>
       </c>
       <c r="C24" s="2">
@@ -5319,7 +5334,7 @@
       <c r="A21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="17" t="s">
         <v>83</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -6341,7 +6356,7 @@
       <c r="A36" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="16" t="s">
+      <c r="B36" s="17" t="s">
         <v>100</v>
       </c>
       <c r="C36" s="2">
@@ -6414,15 +6429,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AL7"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6"/>
   <cols>
     <col min="9" max="9" width="10.3076923076923" customWidth="1"/>
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
-    <col min="11" max="26" width="20" customWidth="1"/>
+    <col min="11" max="28" width="20" customWidth="1"/>
+    <col min="29" max="29" width="21.1538461538462" customWidth="1"/>
+    <col min="30" max="34" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:38">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6500,31 +6517,43 @@
         <v>103</v>
       </c>
       <c r="AA1" s="11" t="s">
-        <v>5</v>
+        <v>104</v>
       </c>
       <c r="AB1" s="11" t="s">
-        <v>5</v>
+        <v>104</v>
       </c>
       <c r="AC1" s="11" t="s">
-        <v>5</v>
+        <v>104</v>
       </c>
       <c r="AD1" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="AE1" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="AE1" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AF1" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AG1" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AH1" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AI1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AF1" s="7" t="s">
+      <c r="AJ1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AG1" s="7" t="s">
+      <c r="AK1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="AH1" s="7" t="s">
+      <c r="AL1" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:34">
+    <row r="2" spans="1:38">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -6555,7 +6584,7 @@
       <c r="J2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="13" t="s">
         <v>9</v>
       </c>
       <c r="L2" s="7" t="s">
@@ -6615,25 +6644,29 @@
       <c r="AD2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="AE2" s="7" t="s">
+      <c r="AE2" s="12"/>
+      <c r="AF2" s="12"/>
+      <c r="AG2" s="12"/>
+      <c r="AH2" s="12"/>
+      <c r="AI2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="AF2" s="7" t="s">
+      <c r="AJ2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="AG2" s="7" t="s">
+      <c r="AK2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="AH2" s="7" t="s">
+      <c r="AL2" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:34">
+    <row r="3" spans="1:38">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>20</v>
@@ -6655,14 +6688,14 @@
       <c r="J3" s="5">
         <v>0</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="K3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M3" s="7"/>
-      <c r="N3" s="13" t="s">
+      <c r="N3" s="14" t="s">
         <v>20</v>
       </c>
       <c r="O3" s="8">
@@ -6672,7 +6705,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="8"/>
-      <c r="R3" s="14">
+      <c r="R3" s="15">
         <v>0</v>
       </c>
       <c r="S3" s="9" t="s">
@@ -6692,7 +6725,7 @@
         <v>1</v>
       </c>
       <c r="Y3" s="10"/>
-      <c r="Z3" s="15">
+      <c r="Z3" s="16">
         <v>0</v>
       </c>
       <c r="AA3" s="11">
@@ -6702,28 +6735,32 @@
         <v>1</v>
       </c>
       <c r="AC3" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="AD3" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="12"/>
+      <c r="AF3" s="12"/>
+      <c r="AG3" s="12"/>
+      <c r="AH3" s="12"/>
+      <c r="AI3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK3" s="7"/>
+      <c r="AL3" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38">
+      <c r="A4" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AD3" s="11">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AG3" s="7"/>
-      <c r="AH3" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:34">
-      <c r="A4" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="B4" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -6745,14 +6782,14 @@
       <c r="J4" s="5">
         <v>0</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="13" t="s">
         <v>20</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M4" s="7"/>
-      <c r="N4" s="13" t="s">
+      <c r="N4" s="14" t="s">
         <v>20</v>
       </c>
       <c r="O4" s="8">
@@ -6762,7 +6799,7 @@
         <v>1</v>
       </c>
       <c r="Q4" s="8"/>
-      <c r="R4" s="14">
+      <c r="R4" s="15">
         <v>0</v>
       </c>
       <c r="S4" s="9" t="s">
@@ -6782,7 +6819,7 @@
         <v>1</v>
       </c>
       <c r="Y4" s="10"/>
-      <c r="Z4" s="15">
+      <c r="Z4" s="16">
         <v>0</v>
       </c>
       <c r="AA4" s="11">
@@ -6795,23 +6832,27 @@
       <c r="AD4" s="11">
         <v>0</v>
       </c>
-      <c r="AE4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AG4" s="7"/>
-      <c r="AH4" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:34">
+      <c r="AE4" s="12"/>
+      <c r="AF4" s="12"/>
+      <c r="AG4" s="12"/>
+      <c r="AH4" s="12"/>
+      <c r="AI4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK4" s="7"/>
+      <c r="AL4" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38">
       <c r="A5" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>20</v>
@@ -6833,14 +6874,14 @@
       <c r="J5" s="5">
         <v>0</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="K5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M5" s="7"/>
-      <c r="N5" s="13" t="s">
+      <c r="N5" s="14" t="s">
         <v>20</v>
       </c>
       <c r="O5" s="8">
@@ -6850,7 +6891,7 @@
         <v>1</v>
       </c>
       <c r="Q5" s="8"/>
-      <c r="R5" s="14">
+      <c r="R5" s="15">
         <v>0</v>
       </c>
       <c r="S5" s="9" t="s">
@@ -6870,7 +6911,7 @@
         <v>1</v>
       </c>
       <c r="Y5" s="10"/>
-      <c r="Z5" s="15">
+      <c r="Z5" s="16">
         <v>0</v>
       </c>
       <c r="AA5" s="11">
@@ -6883,23 +6924,27 @@
       <c r="AD5" s="11">
         <v>0</v>
       </c>
-      <c r="AE5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AG5" s="7"/>
-      <c r="AH5" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:34">
+      <c r="AE5" s="12"/>
+      <c r="AF5" s="12"/>
+      <c r="AG5" s="12"/>
+      <c r="AH5" s="12"/>
+      <c r="AI5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK5" s="7"/>
+      <c r="AL5" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:38">
       <c r="A6" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -6921,14 +6966,14 @@
       <c r="J6" s="5">
         <v>0</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="K6" s="13" t="s">
         <v>20</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M6" s="7"/>
-      <c r="N6" s="13" t="s">
+      <c r="N6" s="14" t="s">
         <v>20</v>
       </c>
       <c r="O6" s="8">
@@ -6938,7 +6983,7 @@
         <v>1</v>
       </c>
       <c r="Q6" s="8"/>
-      <c r="R6" s="14">
+      <c r="R6" s="15">
         <v>0</v>
       </c>
       <c r="S6" s="9" t="s">
@@ -6958,7 +7003,7 @@
         <v>1</v>
       </c>
       <c r="Y6" s="10"/>
-      <c r="Z6" s="15">
+      <c r="Z6" s="16">
         <v>0</v>
       </c>
       <c r="AA6" s="11">
@@ -6971,20 +7016,24 @@
       <c r="AD6" s="11">
         <v>0</v>
       </c>
-      <c r="AE6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AG6" s="7"/>
-      <c r="AH6" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:34">
+      <c r="AE6" s="12"/>
+      <c r="AF6" s="12"/>
+      <c r="AG6" s="12"/>
+      <c r="AH6" s="12"/>
+      <c r="AI6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK6" s="7"/>
+      <c r="AL6" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:38">
       <c r="A7" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>
@@ -7009,14 +7058,14 @@
       <c r="J7" s="5">
         <v>0</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="13" t="s">
         <v>20</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M7" s="7"/>
-      <c r="N7" s="13" t="s">
+      <c r="N7" s="14" t="s">
         <v>20</v>
       </c>
       <c r="O7" s="8">
@@ -7026,7 +7075,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="8"/>
-      <c r="R7" s="14">
+      <c r="R7" s="15">
         <v>0</v>
       </c>
       <c r="S7" s="9" t="s">
@@ -7046,7 +7095,7 @@
         <v>1</v>
       </c>
       <c r="Y7" s="10"/>
-      <c r="Z7" s="15">
+      <c r="Z7" s="16">
         <v>0</v>
       </c>
       <c r="AA7" s="11">
@@ -7059,14 +7108,18 @@
       <c r="AD7" s="11">
         <v>0</v>
       </c>
-      <c r="AE7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AG7" s="7"/>
-      <c r="AH7" s="7" t="s">
+      <c r="AE7" s="12"/>
+      <c r="AF7" s="12"/>
+      <c r="AG7" s="12"/>
+      <c r="AH7" s="12"/>
+      <c r="AI7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK7" s="7"/>
+      <c r="AL7" s="7" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-06-12 09:40:04
</commit_message>
<xml_diff>
--- a/智慧招采平台/过程文件/项目立项字段表.xlsx
+++ b/智慧招采平台/过程文件/项目立项字段表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15020" activeTab="2"/>
+    <workbookView windowHeight="15100" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="113">
   <si>
     <t>招标方式</t>
   </si>
@@ -347,7 +347,10 @@
     <t>直接采购（公开）</t>
   </si>
   <si>
-    <t>直接采购（邀请）</t>
+    <t>竞价（公开）</t>
+  </si>
+  <si>
+    <t>竞价（邀请）</t>
   </si>
   <si>
     <t>邀请供应商</t>
@@ -531,7 +534,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -577,12 +580,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -946,7 +943,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -970,16 +967,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -988,85 +985,85 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1107,8 +1104,8 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6436,7 +6433,10 @@
     <col min="10" max="10" width="12.7692307692308" customWidth="1"/>
     <col min="11" max="28" width="20" customWidth="1"/>
     <col min="29" max="29" width="21.1538461538462" customWidth="1"/>
-    <col min="30" max="34" width="20" customWidth="1"/>
+    <col min="30" max="30" width="20" customWidth="1"/>
+    <col min="31" max="36" width="15.1538461538462" customWidth="1"/>
+    <col min="37" max="37" width="21.1538461538462" customWidth="1"/>
+    <col min="38" max="38" width="15.1538461538462" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -6528,29 +6528,29 @@
       <c r="AD1" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="AE1" s="12" t="s">
+      <c r="AE1" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="AF1" s="12" t="s">
+      <c r="AF1" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="AG1" s="12" t="s">
+      <c r="AG1" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="AH1" s="12" t="s">
+      <c r="AH1" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="AI1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AL1" s="7" t="s">
-        <v>6</v>
+      <c r="AI1" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ1" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="AK1" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="AL1" s="12" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:38">
@@ -6644,29 +6644,37 @@
       <c r="AD2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="AE2" s="12"/>
-      <c r="AF2" s="12"/>
-      <c r="AG2" s="12"/>
-      <c r="AH2" s="12"/>
-      <c r="AI2" s="7" t="s">
+      <c r="AE2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="AJ2" s="7" t="s">
+      <c r="AF2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="AK2" s="7" t="s">
+      <c r="AG2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="AL2" s="7" t="s">
+      <c r="AH2" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="AI2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="AK2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL2" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:38">
       <c r="A3" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>20</v>
@@ -6735,32 +6743,40 @@
         <v>1</v>
       </c>
       <c r="AC3" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AD3" s="11">
         <v>0</v>
       </c>
-      <c r="AE3" s="12"/>
-      <c r="AF3" s="12"/>
-      <c r="AG3" s="12"/>
-      <c r="AH3" s="12"/>
-      <c r="AI3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AK3" s="7"/>
-      <c r="AL3" s="7" t="s">
-        <v>20</v>
+      <c r="AE3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI3" s="8">
+        <v>1</v>
+      </c>
+      <c r="AJ3" s="8">
+        <v>1</v>
+      </c>
+      <c r="AK3" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="AL3" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:38">
       <c r="A4" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -6832,27 +6848,33 @@
       <c r="AD4" s="11">
         <v>0</v>
       </c>
-      <c r="AE4" s="12"/>
-      <c r="AF4" s="12"/>
-      <c r="AG4" s="12"/>
-      <c r="AH4" s="12"/>
-      <c r="AI4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AK4" s="7"/>
-      <c r="AL4" s="7" t="s">
-        <v>20</v>
+      <c r="AE4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI4" s="8">
+        <v>1</v>
+      </c>
+      <c r="AJ4" s="8">
+        <v>1</v>
+      </c>
+      <c r="AK4" s="8"/>
+      <c r="AL4" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:38">
       <c r="A5" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>20</v>
@@ -6924,27 +6946,33 @@
       <c r="AD5" s="11">
         <v>0</v>
       </c>
-      <c r="AE5" s="12"/>
-      <c r="AF5" s="12"/>
-      <c r="AG5" s="12"/>
-      <c r="AH5" s="12"/>
-      <c r="AI5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AK5" s="7"/>
-      <c r="AL5" s="7" t="s">
-        <v>20</v>
+      <c r="AE5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI5" s="8">
+        <v>1</v>
+      </c>
+      <c r="AJ5" s="8">
+        <v>1</v>
+      </c>
+      <c r="AK5" s="8"/>
+      <c r="AL5" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:38">
       <c r="A6" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>20</v>
@@ -7016,24 +7044,30 @@
       <c r="AD6" s="11">
         <v>0</v>
       </c>
-      <c r="AE6" s="12"/>
-      <c r="AF6" s="12"/>
-      <c r="AG6" s="12"/>
-      <c r="AH6" s="12"/>
-      <c r="AI6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AK6" s="7"/>
-      <c r="AL6" s="7" t="s">
-        <v>20</v>
+      <c r="AE6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI6" s="8">
+        <v>1</v>
+      </c>
+      <c r="AJ6" s="8">
+        <v>1</v>
+      </c>
+      <c r="AK6" s="8"/>
+      <c r="AL6" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:38">
       <c r="A7" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>47</v>
@@ -7108,19 +7142,25 @@
       <c r="AD7" s="11">
         <v>0</v>
       </c>
-      <c r="AE7" s="12"/>
-      <c r="AF7" s="12"/>
-      <c r="AG7" s="12"/>
-      <c r="AH7" s="12"/>
-      <c r="AI7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AJ7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="AK7" s="7"/>
-      <c r="AL7" s="7" t="s">
-        <v>20</v>
+      <c r="AE7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI7" s="8">
+        <v>1</v>
+      </c>
+      <c r="AJ7" s="8">
+        <v>1</v>
+      </c>
+      <c r="AK7" s="8"/>
+      <c r="AL7" s="8">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>